<commit_message>
📝 ADD : AFRICA_FR
- 나이지리아 1차 번역작업 완료
</commit_message>
<xml_diff>
--- a/ai-gate/copy.xlsx
+++ b/ai-gate/copy.xlsx
@@ -3,20 +3,21 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="10315"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ABF6FE0F-7A9C-6749-822F-A59FA0F3B651}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{404349CD-B0A3-9242-8DB7-9C06B6A7E81A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="34560" windowHeight="21580" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="34560" windowHeight="21580" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="sample" sheetId="1" r:id="rId1"/>
     <sheet name="LEVANT_AR" sheetId="2" r:id="rId2"/>
+    <sheet name="AFRICA_FR" sheetId="4" r:id="rId3"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="660" uniqueCount="151">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="961" uniqueCount="242">
   <si>
     <t>Type</t>
   </si>
@@ -490,12 +491,398 @@
     <t>ssss</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
+  <si>
+    <t>Une femme passe et la lumière s'allume automatiquement. La phrase ''Sensation intelligente'' apparaît à l'écran.
+Un homme et une femme s'embrassent tandis que l'enceinte XBOOM s'active, accompagnée de la phrase ''Compréhension profonde''.
+Un homme est assis tristement au volant. Le logo LG AI apparaît avec la phrase ''Attention chaleureuse''.
+Un match de football est diffusé à la télévision. L'IA LG répond par une interaction vocale. La phrase ''Pour une vie agréable'' apparaît ci-dessous.
+XBOOM, la télévision et une famille assise sur le canapé avec leur chien apparaissent dans un seul cadre.
+Une mère et son fils utilisent la machine à laver ensemble. La phrase ''Pour une vie facile'' apparaît.
+Des scènes de la mère et du fils, un gros plan sur le bouton AI Wash et un homme utilisant l'ordinateur portable LG Gram sont superposées sur un seul plan, avec la phrase ''Pour une vie facile''.
+Un homme et une femme sont assis à l'avant d'une voiture. Le logo LG AI apparaît entre eux, accompagné de la phrase ''Pour votre puits''. Une vie bienveillante.
+Une personne entre dans un bureau avec son chien. Le purificateur d'air se met en marche.
+Plan final : un fond blanc avec le logo LG AI et la phrase ''Votre Allié Intelligent''.</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>LG AI logo</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Chez LG, nous nous sommes demandés : à quoi sert l'IA ? &lt;br&gt;
+              Après mûre réflexion, nous avons trouvé la réponse. &lt;br&gt;&lt;br&gt;
+              Pour nous, l'IA va au-delà de l'Intelligence Artificielle, c'est une Intelligence Affectueuse. &lt;br&gt;&lt;br&gt;
+              A mesure qu'elle s'intègre à notre quotidien, &lt;br&gt;
+              elle doit contribuer à améliorer notre quotidien. &lt;br&gt;&lt;br&gt;
+              C'est pourquoi VOUS êtes au centre de notre réfléxion.
+              &lt;strong&gt;Découvrez Life's Good avec LG AI&lt;/strong&gt;</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Une vie merveilleuse</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Pour votre vie merveilleuse</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Un homme et une femme sont assis sur le canapé et regardent un match de foot sur un téléviseur LG dans le salon. La scène change et l'homme et la femme s'enlacent. La caméra se concentre sur la LG XBOOM à côté d'eux.</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>LG AI comprend votre vie et améliore vos expériences pour rendre votre vie remplie de moments agréables.</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Une vie sans effort</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Une vie bien soignée</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Apprendre Encore Plus</t>
+  </si>
+  <si>
+    <t>Vue de face du produit LG OLED evo AI</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Vue de face du produit LG OLED  AI</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>https://www.lg.com/africa_fr/television/lg-oled83c56la</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>https://www.lg.com/africa_fr/oled-tvs</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>https://www.lg.com/africa_fr/qned-tvs</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>https://www.lg.com/africa_fr/nanocell-tvs</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Vue de face du produit LG Nanocell  AI</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Une mère et son fils utilisent ensemble une machine à laver LG AI, tournant le cadran pour activer AI Wash. Un homme utilisant l'ordinateur portable LG gram apparaît dans la même séquence.</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Pour votre vie sans effort</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>https://www.lg.com/africa_fr/washing-machines/lg-wt1310rh</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Vue de face du produit LG WashTower AI</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>https://www.lg.com/africa_fr/washing-machines/lg-f0l9dgp2s</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>https://www.lg.com/africa_fr/refrigerators/lg-gc-x24ffcab</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Vue de face du produit LG InstaView AI</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>LG AI prend soin de vous, de votre espace et de la planète pour rendre votre vie bien entretenue, comme vous le désirez.</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Un homme entre dans le bureau, tenant un chien en laisse. L'homme au volant a l'air triste tandis que l'IA LG lui montre une photo de famille. L'écran de la voiture s'affiche en gros plan tandis que l'IA LG affiche une carte et revisite un souvenir.</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>https://www.lg.com/global/mobility/mobility-labworks-series/adas-solutions/in-cabin-vision</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Utilisateur interagissant avec l'interface à écran tactile alimentée par une solution IHM IA multimodale, sélectionnant le menu du café avec l'invite de l'assistant IA</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>https://www.lg.com/global/mobility/mobility-labworks-series/digital-cockpit-solutions/digital-cockpit-gamma</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Climatisation</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Appareils électroménagers</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Le téléviseur LG AI apprend vos préférences de visionnage et comprend votre style de vie pour optimiser chaque aspect de votre expérience télévisuelle, créant ainsi un divertissement personnalisé idéal rien que pour vous.</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t xml:space="preserve">téléviseur LG AI </t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Découvrez la nouvelle génération de&lt;br&gt;
+                          téléviseurs LG AI</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>https://www.lg.com/africa_fr/television/ai-tv</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Sur l'écran d'un téléviseur LG OLED, la page d'accueil webOS 25 regorge d'applications et de contenus de divertissement. À côté du téléviseur se trouve la télécommande LG AI Magic ; le bouton IA est mis en surbrillance comme s'il était activé par la voix. Une bulle de dialogue apparaît à côté : ''Suggérer un film que j'aime".</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Écran de téléviseur LG OLED montrant le fonctionnement de la recherche IA. Une petite fenêtre de discussion s'ouvre, montrant comment l'utilisateur a demandé quels jeux de sport étaient disponibles. La recherche IA a répondu par chat et en affichant des vignettes des différents contenus disponibles. Une invite permet également de demander à Microsoft Copilot.</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>La télécommande LG AI Magic en action. Une brève pression sur le bouton AI active l'assistant IA sur l'écran du téléviseur OLED, qui suggère ensuite des mots-clés.</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Un contenu de science-fiction est diffusé sur un téléviseur OLED LG. À gauche de l'écran se trouve l'interface du chatbot IA. L'utilisateur signale au chatbot que l'écran est trop sombre et celui-ci propose des solutions.</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Femme chantant dans un microphone avec un casque, mise en valeur par l'amélioration du son du processeur LG α11 AI</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Deux scènes connectées avec la télécommande LG AI Magic Remote devant un téléviseur : la première montrant une scène de science-fiction, la seconde montrant un écran d'accueil avec du contenu personnalisé</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>*Les fonctionnalités d'IA de LG utilisent des algorithmes entraînés par l'apprentissage profond pour la mise à l'échelle de l'image et le mixage audio en temps réel.</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>**Tous les téléviseurs LG webOS 24 sont dotés de la personnalisation par IA, à l'exception de ceux sans capteur de lumière.</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>&lt;img src="./assets/image/ai-product-category-audio-eyebrow-logo-desktop.svg" alt="Audio" class="eyebrow-logo" loading="lazy" data-tp="alt"&gt;
+                      Cela semble particulièrement juste</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>&lt;img src="./assets/image/ai-product-category-tv-eyebrow-logo-desktop.svg" alt="TV" class="eyebrow-logo" loading="lazy" data-tp="alt"&gt;
+                      Évolue pour satisfaire tous vos besoins de divertissement</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>LG xboom AI analyse et ajuste le son en fonction du genre et de l'espace. Grâce à l'éclairage IA qui sublime l'ambiance et s'harmonise avec votre musique, vous profitez d'un son et d'une ambiance uniques.</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Une femme et un homme s'embrassent dans le salon, avec l'enceinte XBOOM allumée à côté d'eux.</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Profitez d'une nouvelle expérience sonore &lt;br&gt;
+                          avec LG xboom AI</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Enceinte LG XBOOM avec modes sonores IA, notamment Bass Boost, Voice Enhance et Standard</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Enceinte LG XBOOM avec éclairage IA qui s'adapte aux modes voix, ambiance et fête</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Enceinte LG XBOOM placée sur une table dans une pièce aux tons rouges avec des murs à motifs quadrillés et des meubles modernes</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>&lt;img src="./assets/image/ai-product-category-appliances-eyebrow-logo-desktop.svg" alt="Appareils électroménagers" class="eyebrow-logo" loading="lazy" data-tp="alt"&gt;
+                      Allégez toutes vos charges</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>LG WashTower AI détecte ce que vous lavez pour fournir un lavage optimisé pour le soin des tissus sensibles, vous assurant ainsi de perfectionner sans effort chaque charge, à chaque fois.</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Découvrez un nouveau mode de vie &lt;br&gt;
+                          avec LG AI Core Tech</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Laveuse et sécheuse superposées LG intégrées dans une buanderie moderne avec armoires en bois et banquette</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Réglage manuel du cycle de lavage AI sur la machine à laver LG à l'aide du cadran de commande intelligent</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>L'utilisateur sélectionne le cycle de séchage AI sur le sèche-linge LG à l'aide du cadran de commande numérique</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>*Ce produit sera commercialisé progressivement dans certains pays.</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>**La détection IA est activée lorsque la charge est inférieure à 6 kg.</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>***Le lavage IA doit être utilisé uniquement avec des tissus similaires [tous les tissus ne sont pas détectés] et une lessive adaptée.</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>****Le séchage IA est disponible uniquement pour les charges inférieures à 5 kg avec des tissus présentant le même niveau d'absorption d'humidité. »</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>&lt;img src="./assets/image/ai-product-category-air-conditioning-eyebrow-logo-desktop.svg" alt="Climatisation" class="eyebrow-logo" loading="lazy" data-tp="alt"&gt;
+                      Confort avec un refroidissement parfaitement réglé</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>LG DUALCOOL AI assure une qualité d'air optimale pour votre confort tout en optimisant l'efficacité énergétique pour vous aider à réduire vos coûts. Avec LG AI Air, profitez d'une climatisation parfaitement adaptée à votre confort.</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Découvrez un confort optimisé &lt;br&gt;
+                          avec LG AI Air</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Le climatiseur LG DUAL Inverter refroidit un salon moderne, où une femme est assise sur le canapé, alimenté par la technologie ThinQ AI.</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Une femme se détend dans un salon intelligent tandis que le climatiseur LG AI ajuste automatiquement la température, le débit d'air et l'humidité</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Interface smartphone affichant un graphique de consommation d'énergie devant le climatiseur LG, mettant en évidence AI kW Manager pour une surveillance efficace de la puissance</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>*L'AI Air peut être commandé via une télécommande et ThinQ.</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>**L'AI Air est disponible en modes refroidissement et chauffage.</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>***Lors de l'utilisation de l'AI Air, le volume d'air et la direction du vent s'ajustent automatiquement en fonction de la situation, et l'AI Air se désactive lorsque la direction du vent change.</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>****Lorsque l'AI Air est activé, le capteur radar détecte la position de l'occupant et active automatiquement le vent direct/indirect.</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>*****La distance de détection du capteur radar peut atteindre 5 m, et des différences peuvent survenir selon l'installation et l'environnement d'utilisation du produit.</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>*****Cette fonction est uniquement compatible avec les modèles équipés de capteurs radar.</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>ThinQ® vous aide à réaliser votre vie</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Plateforme pour vos appareils et appareils intelligents LG, ThinQ met le contrôle et la commodité à portée de main, pour vous aider à simplifier la vie et à profiter du confort de la maison.</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>https://www.lg.com/africa_fr/lg-thinq</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Une personne tient un smartphone avec l'application LG ThinQ ouverte, gérant des appareils domestiques intelligents tout en buvant du café.</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Dans une cuisine intelligente moderne, une femme utilise une commande vocale pour démarrer la machine à laver avec LG ThinQ AI, tandis qu'un homme lit sur le canapé en arrière-plan.</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Contrôle simple avec l'assistant vocal</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Dites à votre appareil LG exactement ce dont vous avez besoin en le disant simplement, et le haut-parleur IA écoutera et vérifiera le cycle pour vous le faire savoir.</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Un smartphone affiche l'application LG ThinQ contrôlant le four coulissant LG InstaView, permettant un entretien efficace des produits dans la cuisine.</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Maintenance efficace des produits</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Grâce à l'application LG ThinQ, vérifiez votre appareil LG, téléchargez de nouveaux cycles, surveillez l'utilisation des cycles et bien plus encore.</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>En savoir plus sur LG Affectionate Intelligence</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Un dirigeant de LG Electronics détient un certificat d'accréditation en cybersécurité, avec un graphique de sécurité numérique en arrière-plan</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>LG renforce son leadership en matière de cybersécurité avec l'accréditation KOLAS IoT Cybersecurity Testing</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>https://www.lgnewsroom.com/2025/01/lg-strengthens-cybersecurity-leadership-with-kolas-iot-cybersecurity-testing-accreditation/</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Les visiteurs admirent l'écran LED incurvé de LG arborant le slogan « Life's Good 24/7 » lors d'une exposition technologique</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>LG présente ses dernières innovations, propulsées par « Affectionate Intelligence », au CES 2025</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Intervenant présentant des solutions B2B basées sur l'IA sur scène lors d'un événement LG</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>LG dévoile une journée dans la vie avec "Affectionate Intelligence'' lors de la première mondiale de LG</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3">
+  <fonts count="4">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -515,6 +902,14 @@
       <name val="맑은 고딕"/>
       <family val="3"/>
       <charset val="129"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
+      <name val="맑은 고딕"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
   </fonts>
@@ -540,15 +935,21 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
     <cellStyle name="표준" xfId="0" builtinId="0"/>
+    <cellStyle name="하이퍼링크" xfId="1" builtinId="8"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -913,7 +1314,7 @@
         <v>4</v>
       </c>
       <c r="B3" t="s">
-        <v>5</v>
+        <v>152</v>
       </c>
     </row>
     <row r="4" spans="1:2">
@@ -3553,4 +3954,1268 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D1CECDB3-77B8-B245-85F1-872FFBD72961}">
+  <dimension ref="A1:B165"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="17"/>
+  <cols>
+    <col min="1" max="1" width="15" customWidth="1"/>
+    <col min="2" max="2" width="120" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" s="1" customFormat="1">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" ht="234">
+      <c r="A2" t="s">
+        <v>2</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2">
+      <c r="A3" t="s">
+        <v>4</v>
+      </c>
+      <c r="B3" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" ht="126">
+      <c r="A4" t="s">
+        <v>2</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2">
+      <c r="A5" t="s">
+        <v>4</v>
+      </c>
+      <c r="B5" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2">
+      <c r="A6" t="s">
+        <v>2</v>
+      </c>
+      <c r="B6" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2">
+      <c r="A7" t="s">
+        <v>2</v>
+      </c>
+      <c r="B7" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2">
+      <c r="A8" t="s">
+        <v>2</v>
+      </c>
+      <c r="B8" t="s">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2">
+      <c r="A9" t="s">
+        <v>2</v>
+      </c>
+      <c r="B9" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2">
+      <c r="A10" t="s">
+        <v>2</v>
+      </c>
+      <c r="B10" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2">
+      <c r="A11" t="s">
+        <v>2</v>
+      </c>
+      <c r="B11" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2">
+      <c r="A12" t="s">
+        <v>14</v>
+      </c>
+      <c r="B12" s="3" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2">
+      <c r="A13" t="s">
+        <v>4</v>
+      </c>
+      <c r="B13" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2">
+      <c r="A14" t="s">
+        <v>2</v>
+      </c>
+      <c r="B14" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2">
+      <c r="A15" t="s">
+        <v>14</v>
+      </c>
+      <c r="B15" s="3" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2">
+      <c r="A16" t="s">
+        <v>4</v>
+      </c>
+      <c r="B16" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2">
+      <c r="A17" t="s">
+        <v>2</v>
+      </c>
+      <c r="B17" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2">
+      <c r="A18" t="s">
+        <v>14</v>
+      </c>
+      <c r="B18" s="3" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2">
+      <c r="A19" t="s">
+        <v>4</v>
+      </c>
+      <c r="B19" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2">
+      <c r="A20" t="s">
+        <v>2</v>
+      </c>
+      <c r="B20" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2">
+      <c r="A21" t="s">
+        <v>14</v>
+      </c>
+      <c r="B21" s="3" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2">
+      <c r="A22" t="s">
+        <v>4</v>
+      </c>
+      <c r="B22" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2">
+      <c r="A23" t="s">
+        <v>2</v>
+      </c>
+      <c r="B23" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2">
+      <c r="A24" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2">
+      <c r="A25" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="26" spans="1:2">
+      <c r="A26" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="27" spans="1:2">
+      <c r="A27" t="s">
+        <v>2</v>
+      </c>
+      <c r="B27" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="28" spans="1:2">
+      <c r="A28" t="s">
+        <v>2</v>
+      </c>
+      <c r="B28" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="29" spans="1:2">
+      <c r="A29" t="s">
+        <v>2</v>
+      </c>
+      <c r="B29" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="30" spans="1:2">
+      <c r="A30" t="s">
+        <v>14</v>
+      </c>
+      <c r="B30" s="3" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="31" spans="1:2">
+      <c r="A31" t="s">
+        <v>4</v>
+      </c>
+      <c r="B31" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="32" spans="1:2">
+      <c r="A32" t="s">
+        <v>2</v>
+      </c>
+      <c r="B32" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="33" spans="1:2">
+      <c r="A33" t="s">
+        <v>14</v>
+      </c>
+      <c r="B33" s="3" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="34" spans="1:2">
+      <c r="A34" t="s">
+        <v>4</v>
+      </c>
+      <c r="B34" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="35" spans="1:2">
+      <c r="A35" t="s">
+        <v>2</v>
+      </c>
+      <c r="B35" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="36" spans="1:2">
+      <c r="A36" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="37" spans="1:2">
+      <c r="A37" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="38" spans="1:2">
+      <c r="A38" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="39" spans="1:2">
+      <c r="A39" t="s">
+        <v>14</v>
+      </c>
+      <c r="B39" s="3" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="40" spans="1:2">
+      <c r="A40" t="s">
+        <v>4</v>
+      </c>
+      <c r="B40" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="41" spans="1:2">
+      <c r="A41" t="s">
+        <v>2</v>
+      </c>
+      <c r="B41" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="42" spans="1:2">
+      <c r="A42" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="43" spans="1:2">
+      <c r="A43" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="44" spans="1:2">
+      <c r="A44" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="45" spans="1:2">
+      <c r="A45" t="s">
+        <v>2</v>
+      </c>
+      <c r="B45" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="46" spans="1:2">
+      <c r="A46" t="s">
+        <v>2</v>
+      </c>
+      <c r="B46" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="47" spans="1:2">
+      <c r="A47" t="s">
+        <v>2</v>
+      </c>
+      <c r="B47" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="48" spans="1:2">
+      <c r="A48" t="s">
+        <v>14</v>
+      </c>
+      <c r="B48" s="3" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="49" spans="1:2">
+      <c r="A49" t="s">
+        <v>4</v>
+      </c>
+      <c r="B49" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="50" spans="1:2">
+      <c r="A50" t="s">
+        <v>2</v>
+      </c>
+      <c r="B50" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="51" spans="1:2">
+      <c r="A51" t="s">
+        <v>14</v>
+      </c>
+      <c r="B51" s="3" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="52" spans="1:2">
+      <c r="A52" t="s">
+        <v>4</v>
+      </c>
+      <c r="B52" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="53" spans="1:2">
+      <c r="A53" t="s">
+        <v>2</v>
+      </c>
+      <c r="B53" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="54" spans="1:2">
+      <c r="A54" t="s">
+        <v>14</v>
+      </c>
+      <c r="B54" s="3" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="55" spans="1:2">
+      <c r="A55" t="s">
+        <v>4</v>
+      </c>
+      <c r="B55" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="56" spans="1:2">
+      <c r="A56" t="s">
+        <v>2</v>
+      </c>
+      <c r="B56" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="57" spans="1:2">
+      <c r="A57" t="s">
+        <v>2</v>
+      </c>
+      <c r="B57" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="58" spans="1:2">
+      <c r="A58" t="s">
+        <v>2</v>
+      </c>
+      <c r="B58" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="59" spans="1:2">
+      <c r="A59" t="s">
+        <v>2</v>
+      </c>
+      <c r="B59" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="60" spans="1:2">
+      <c r="A60" t="s">
+        <v>2</v>
+      </c>
+      <c r="B60" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="61" spans="1:2">
+      <c r="A61" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="62" spans="1:2" ht="54">
+      <c r="A62" t="s">
+        <v>2</v>
+      </c>
+      <c r="B62" s="2" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="63" spans="1:2">
+      <c r="A63" t="s">
+        <v>4</v>
+      </c>
+      <c r="B63" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="64" spans="1:2">
+      <c r="A64" t="s">
+        <v>2</v>
+      </c>
+      <c r="B64" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="65" spans="1:2">
+      <c r="A65" t="s">
+        <v>4</v>
+      </c>
+      <c r="B65" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="66" spans="1:2" ht="36">
+      <c r="A66" t="s">
+        <v>2</v>
+      </c>
+      <c r="B66" s="2" t="s">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="67" spans="1:2">
+      <c r="A67" t="s">
+        <v>2</v>
+      </c>
+      <c r="B67" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="68" spans="1:2">
+      <c r="A68" t="s">
+        <v>14</v>
+      </c>
+      <c r="B68" s="3" t="s">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="69" spans="1:2">
+      <c r="A69" t="s">
+        <v>4</v>
+      </c>
+      <c r="B69" t="s">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="70" spans="1:2">
+      <c r="A70" t="s">
+        <v>2</v>
+      </c>
+      <c r="B70" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="71" spans="1:2">
+      <c r="A71" t="s">
+        <v>4</v>
+      </c>
+      <c r="B71" t="s">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="72" spans="1:2">
+      <c r="A72" t="s">
+        <v>2</v>
+      </c>
+      <c r="B72" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="73" spans="1:2">
+      <c r="A73" t="s">
+        <v>4</v>
+      </c>
+      <c r="B73" t="s">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="74" spans="1:2">
+      <c r="A74" t="s">
+        <v>2</v>
+      </c>
+      <c r="B74" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="75" spans="1:2">
+      <c r="A75" t="s">
+        <v>4</v>
+      </c>
+      <c r="B75" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="76" spans="1:2">
+      <c r="A76" t="s">
+        <v>2</v>
+      </c>
+      <c r="B76" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="77" spans="1:2">
+      <c r="A77" t="s">
+        <v>4</v>
+      </c>
+      <c r="B77" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="78" spans="1:2">
+      <c r="A78" t="s">
+        <v>2</v>
+      </c>
+      <c r="B78" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="79" spans="1:2">
+      <c r="A79" t="s">
+        <v>4</v>
+      </c>
+      <c r="B79" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="80" spans="1:2">
+      <c r="A80" t="s">
+        <v>2</v>
+      </c>
+      <c r="B80" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="81" spans="1:2">
+      <c r="A81" t="s">
+        <v>2</v>
+      </c>
+      <c r="B81" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="82" spans="1:2">
+      <c r="A82" t="s">
+        <v>2</v>
+      </c>
+      <c r="B82" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="83" spans="1:2" ht="54">
+      <c r="A83" t="s">
+        <v>2</v>
+      </c>
+      <c r="B83" s="2" t="s">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="84" spans="1:2">
+      <c r="A84" t="s">
+        <v>4</v>
+      </c>
+      <c r="B84" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="85" spans="1:2">
+      <c r="A85" t="s">
+        <v>2</v>
+      </c>
+      <c r="B85" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="86" spans="1:2">
+      <c r="A86" t="s">
+        <v>4</v>
+      </c>
+      <c r="B86" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="87" spans="1:2" ht="36">
+      <c r="A87" t="s">
+        <v>2</v>
+      </c>
+      <c r="B87" s="2" t="s">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="88" spans="1:2">
+      <c r="A88" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="89" spans="1:2">
+      <c r="A89" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="90" spans="1:2">
+      <c r="A90" t="s">
+        <v>4</v>
+      </c>
+      <c r="B90" t="s">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="91" spans="1:2">
+      <c r="A91" t="s">
+        <v>2</v>
+      </c>
+      <c r="B91" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="92" spans="1:2">
+      <c r="A92" t="s">
+        <v>4</v>
+      </c>
+      <c r="B92" t="s">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="93" spans="1:2">
+      <c r="A93" t="s">
+        <v>2</v>
+      </c>
+      <c r="B93" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="94" spans="1:2">
+      <c r="A94" t="s">
+        <v>4</v>
+      </c>
+      <c r="B94" t="s">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="95" spans="1:2">
+      <c r="A95" t="s">
+        <v>2</v>
+      </c>
+      <c r="B95" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="96" spans="1:2">
+      <c r="A96" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="97" spans="1:2" ht="54">
+      <c r="A97" t="s">
+        <v>2</v>
+      </c>
+      <c r="B97" s="2" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="98" spans="1:2">
+      <c r="A98" t="s">
+        <v>4</v>
+      </c>
+      <c r="B98" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="99" spans="1:2">
+      <c r="A99" t="s">
+        <v>2</v>
+      </c>
+      <c r="B99" t="s">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="100" spans="1:2">
+      <c r="A100" t="s">
+        <v>4</v>
+      </c>
+      <c r="B100" t="s">
+        <v>205</v>
+      </c>
+    </row>
+    <row r="101" spans="1:2" ht="36">
+      <c r="A101" t="s">
+        <v>2</v>
+      </c>
+      <c r="B101" s="2" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="102" spans="1:2">
+      <c r="A102" t="s">
+        <v>2</v>
+      </c>
+      <c r="B102" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="103" spans="1:2">
+      <c r="A103" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="104" spans="1:2">
+      <c r="A104" t="s">
+        <v>4</v>
+      </c>
+      <c r="B104" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="105" spans="1:2">
+      <c r="A105" t="s">
+        <v>2</v>
+      </c>
+      <c r="B105" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="106" spans="1:2">
+      <c r="A106" t="s">
+        <v>4</v>
+      </c>
+      <c r="B106" t="s">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="107" spans="1:2">
+      <c r="A107" t="s">
+        <v>2</v>
+      </c>
+      <c r="B107" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="108" spans="1:2">
+      <c r="A108" t="s">
+        <v>2</v>
+      </c>
+      <c r="B108" t="s">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="109" spans="1:2">
+      <c r="A109" t="s">
+        <v>2</v>
+      </c>
+      <c r="B109" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="110" spans="1:2">
+      <c r="A110" t="s">
+        <v>2</v>
+      </c>
+      <c r="B110" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="111" spans="1:2">
+      <c r="A111" t="s">
+        <v>2</v>
+      </c>
+      <c r="B111" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="112" spans="1:2" ht="54">
+      <c r="A112" t="s">
+        <v>2</v>
+      </c>
+      <c r="B112" s="2" t="s">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="113" spans="1:2">
+      <c r="A113" t="s">
+        <v>4</v>
+      </c>
+      <c r="B113" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="114" spans="1:2">
+      <c r="A114" t="s">
+        <v>2</v>
+      </c>
+      <c r="B114" t="s">
+        <v>213</v>
+      </c>
+    </row>
+    <row r="115" spans="1:2">
+      <c r="A115" t="s">
+        <v>4</v>
+      </c>
+      <c r="B115" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="116" spans="1:2" ht="36">
+      <c r="A116" t="s">
+        <v>2</v>
+      </c>
+      <c r="B116" s="2" t="s">
+        <v>214</v>
+      </c>
+    </row>
+    <row r="117" spans="1:2">
+      <c r="A117" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="118" spans="1:2">
+      <c r="A118" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="119" spans="1:2">
+      <c r="A119" t="s">
+        <v>4</v>
+      </c>
+      <c r="B119" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="120" spans="1:2">
+      <c r="A120" t="s">
+        <v>2</v>
+      </c>
+      <c r="B120" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="121" spans="1:2">
+      <c r="A121" t="s">
+        <v>4</v>
+      </c>
+      <c r="B121" t="s">
+        <v>217</v>
+      </c>
+    </row>
+    <row r="122" spans="1:2">
+      <c r="A122" t="s">
+        <v>2</v>
+      </c>
+      <c r="B122" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="123" spans="1:2">
+      <c r="A123" t="s">
+        <v>2</v>
+      </c>
+      <c r="B123" t="s">
+        <v>218</v>
+      </c>
+    </row>
+    <row r="124" spans="1:2">
+      <c r="A124" t="s">
+        <v>2</v>
+      </c>
+      <c r="B124" t="s">
+        <v>219</v>
+      </c>
+    </row>
+    <row r="125" spans="1:2">
+      <c r="A125" t="s">
+        <v>2</v>
+      </c>
+      <c r="B125" t="s">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="126" spans="1:2">
+      <c r="A126" t="s">
+        <v>2</v>
+      </c>
+      <c r="B126" t="s">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="127" spans="1:2">
+      <c r="A127" t="s">
+        <v>2</v>
+      </c>
+      <c r="B127" t="s">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="128" spans="1:2">
+      <c r="A128" t="s">
+        <v>2</v>
+      </c>
+      <c r="B128" t="s">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="129" spans="1:2">
+      <c r="A129" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="130" spans="1:2">
+      <c r="A130" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="131" spans="1:2">
+      <c r="A131" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="132" spans="1:2">
+      <c r="A132" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="133" spans="1:2">
+      <c r="A133" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="134" spans="1:2">
+      <c r="A134" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="135" spans="1:2">
+      <c r="A135" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="136" spans="1:2">
+      <c r="A136" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="137" spans="1:2">
+      <c r="A137" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="138" spans="1:2">
+      <c r="A138" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="139" spans="1:2">
+      <c r="A139" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="140" spans="1:2">
+      <c r="A140" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="141" spans="1:2">
+      <c r="A141" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="142" spans="1:2">
+      <c r="A142" t="s">
+        <v>2</v>
+      </c>
+      <c r="B142" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="143" spans="1:2">
+      <c r="A143" t="s">
+        <v>2</v>
+      </c>
+      <c r="B143" t="s">
+        <v>225</v>
+      </c>
+    </row>
+    <row r="144" spans="1:2">
+      <c r="A144" t="s">
+        <v>2</v>
+      </c>
+      <c r="B144" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="145" spans="1:2">
+      <c r="A145" t="s">
+        <v>14</v>
+      </c>
+      <c r="B145" s="3" t="s">
+        <v>226</v>
+      </c>
+    </row>
+    <row r="146" spans="1:2">
+      <c r="A146" t="s">
+        <v>4</v>
+      </c>
+      <c r="B146" t="s">
+        <v>227</v>
+      </c>
+    </row>
+    <row r="147" spans="1:2">
+      <c r="A147" t="s">
+        <v>4</v>
+      </c>
+      <c r="B147" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="148" spans="1:2">
+      <c r="A148" t="s">
+        <v>2</v>
+      </c>
+      <c r="B148" t="s">
+        <v>229</v>
+      </c>
+    </row>
+    <row r="149" spans="1:2">
+      <c r="A149" t="s">
+        <v>2</v>
+      </c>
+      <c r="B149" t="s">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="150" spans="1:2">
+      <c r="A150" t="s">
+        <v>4</v>
+      </c>
+      <c r="B150" t="s">
+        <v>231</v>
+      </c>
+    </row>
+    <row r="151" spans="1:2">
+      <c r="A151" t="s">
+        <v>2</v>
+      </c>
+      <c r="B151" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="152" spans="1:2">
+      <c r="A152" t="s">
+        <v>2</v>
+      </c>
+      <c r="B152" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="153" spans="1:2">
+      <c r="A153" t="s">
+        <v>2</v>
+      </c>
+      <c r="B153" t="s">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="154" spans="1:2">
+      <c r="A154" t="s">
+        <v>4</v>
+      </c>
+      <c r="B154" t="s">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="155" spans="1:2">
+      <c r="A155" t="s">
+        <v>2</v>
+      </c>
+      <c r="B155" t="s">
+        <v>236</v>
+      </c>
+    </row>
+    <row r="156" spans="1:2">
+      <c r="A156" t="s">
+        <v>2</v>
+      </c>
+      <c r="B156" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="157" spans="1:2">
+      <c r="A157" t="s">
+        <v>14</v>
+      </c>
+      <c r="B157" s="3" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="158" spans="1:2">
+      <c r="A158" t="s">
+        <v>4</v>
+      </c>
+      <c r="B158" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="159" spans="1:2">
+      <c r="A159" t="s">
+        <v>2</v>
+      </c>
+      <c r="B159" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="160" spans="1:2">
+      <c r="A160" t="s">
+        <v>2</v>
+      </c>
+      <c r="B160" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="161" spans="1:2">
+      <c r="A161" t="s">
+        <v>14</v>
+      </c>
+      <c r="B161" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="162" spans="1:2">
+      <c r="A162" t="s">
+        <v>4</v>
+      </c>
+      <c r="B162" t="s">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="163" spans="1:2">
+      <c r="A163" t="s">
+        <v>2</v>
+      </c>
+      <c r="B163" t="s">
+        <v>241</v>
+      </c>
+    </row>
+    <row r="164" spans="1:2">
+      <c r="A164" t="s">
+        <v>2</v>
+      </c>
+      <c r="B164" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="165" spans="1:2">
+      <c r="A165" t="s">
+        <v>14</v>
+      </c>
+      <c r="B165" t="s">
+        <v>147</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="2" type="noConversion"/>
+  <hyperlinks>
+    <hyperlink ref="B12" r:id="rId1" xr:uid="{F43A1E02-44B8-3642-A3AF-A032972319BB}"/>
+    <hyperlink ref="B15" r:id="rId2" xr:uid="{BDAD240A-8C87-0042-8EAD-BE09CE537A45}"/>
+    <hyperlink ref="B18" r:id="rId3" xr:uid="{992A67C6-2A4A-AC41-A937-1C273FF25DE9}"/>
+    <hyperlink ref="B21" r:id="rId4" xr:uid="{E5660A9B-B304-4B45-B02F-0075BBF31DFF}"/>
+    <hyperlink ref="B30" r:id="rId5" xr:uid="{A908065C-B2FA-E743-B3C8-8AE701A9666B}"/>
+    <hyperlink ref="B33" r:id="rId6" xr:uid="{87730795-4A89-3040-97E0-8E1D8B65BAD5}"/>
+    <hyperlink ref="B39" r:id="rId7" xr:uid="{AC67B0C6-A78B-5F46-B03D-C18D4E1D894B}"/>
+    <hyperlink ref="B48" r:id="rId8" xr:uid="{55E33A50-7572-924C-A799-E340AD254DDE}"/>
+    <hyperlink ref="B54" r:id="rId9" xr:uid="{F2E7B405-77FD-5946-9AAB-40A95243C884}"/>
+    <hyperlink ref="B51" r:id="rId10" xr:uid="{0C9C4D40-8F39-2F45-B499-549596017A90}"/>
+    <hyperlink ref="B68" r:id="rId11" xr:uid="{DC33F75E-1728-4041-9C09-C8631C4069F6}"/>
+    <hyperlink ref="B145" r:id="rId12" xr:uid="{6B263608-70DE-BA46-9EE6-09951BD7527B}"/>
+    <hyperlink ref="B157" r:id="rId13" xr:uid="{5645AD79-F4FC-0C48-BD64-925171F4A3B8}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
📝 ADD : LG AI(SK)
- 번역작업
</commit_message>
<xml_diff>
--- a/ai-gate/copy.xlsx
+++ b/ai-gate/copy.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="10727"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C772067C-99E9-484A-8429-ABC552EEC542}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EC172FE6-AE50-E24D-AC0A-BDF6AD20994E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="34560" windowHeight="21580" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="34560" windowHeight="21580" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="sample" sheetId="1" r:id="rId1"/>
@@ -13,13 +13,14 @@
     <sheet name="AFRICA_FR" sheetId="4" r:id="rId3"/>
     <sheet name="BE_FR" sheetId="5" r:id="rId4"/>
     <sheet name="TN_FR" sheetId="6" r:id="rId5"/>
+    <sheet name="SK" sheetId="8" r:id="rId6"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1506" uniqueCount="476">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1809" uniqueCount="575">
   <si>
     <t>Type</t>
   </si>
@@ -23987,12 +23988,3626 @@
                       Powers everything you do</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
+  <si>
+    <r>
+      <t>Ke</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="238"/>
+      </rPr>
+      <t>ď</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="맑은 고딕"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> sa automaticky rozsvieti svetlo, okolo prechádza žena. Na obrazovke sa objaví veta „Múdro vníma</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="238"/>
+      </rPr>
+      <t>ť</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="맑은 고딕"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>“.
+Muž a žena sa objímajú, ke</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="238"/>
+      </rPr>
+      <t>ď</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="맑은 고딕"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> sa aktivuje reproduktor XBOOM, sprevádzaný frázou „“Hlboké porozumenie".
+Muž sedí smutne na sedadle vodi</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="238"/>
+      </rPr>
+      <t>č</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="맑은 고딕"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>a. Zobrazí sa logo umelej inteligencie LG s frázou „Starostlivo a srde</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="238"/>
+      </rPr>
+      <t>č</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="맑은 고딕"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>ne“ LG AI reaguje hlasovou interakciou. Nižšie sa zobrazí fráza „Pre váš úžasný život“.
+XBOOM, televízor a rodina sediaca na pohovke so psom sa zobrazia v jednom zábere.
+Matka a syn spolo</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="238"/>
+      </rPr>
+      <t>č</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="맑은 고딕"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>ne používajú prá</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="238"/>
+      </rPr>
+      <t>č</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="맑은 고딕"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>ku. Zobrazí sa fráza „Pre váš život bez námahy“.
+Scény matky a syna, detailný záber na voli</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="238"/>
+      </rPr>
+      <t>č</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="맑은 고딕"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> AI Wash a muža používajúceho notebook LG gram sú prekryté do jedného záberu s frázou ,,Pre váš život bez námahy".
+Muž a žena sedia na predných sedadlách auta. Medzi nimi sa zobrazuje logo LG AI spolu s frázou „Pre váš dobrý život“.
+Osoba vchádza do kancelárie so svojím psom. V reakcii na to sa zapne </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="238"/>
+      </rPr>
+      <t>č</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="맑은 고딕"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>isti</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="238"/>
+      </rPr>
+      <t>č</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="맑은 고딕"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>ka vzduchu.
+Závere</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="238"/>
+      </rPr>
+      <t>č</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="맑은 고딕"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>ný záber: biele pozadie s logom LG AI a frázou „Láskavá inteligencia pre VÁS“.</t>
+    </r>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>&lt;span class="gradient-text" data-tp="copy"&gt;Láskavá inteligencia&lt;/span&gt; pre VÁS</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Ikona posúvania nadol</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Nádherný život</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Bezstarostný život</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Spokojný život</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Umelá inteligencia LG rozumie vášmu životu a vylepšuje zážitky, aby bol váš život plný nádherných okamihov.</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t>Muž a žena sedia na pohovke a sledujú v obýva</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="238"/>
+      </rPr>
+      <t>č</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="맑은 고딕"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>ke futbalový prenos na televízore LG . Scéna sa zmení a muž a žena sa objímajú.
+Kamera sa zameria na LG XBOOM ved</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="238"/>
+      </rPr>
+      <t>ľ</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="맑은 고딕"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>a nich.</t>
+    </r>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Zistite viac</t>
+  </si>
+  <si>
+    <t>Pre váš nádherný život</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>https://www.lg.com/sk/televizory/lg-oled55c5elb</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t>Predný poh</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="238"/>
+      </rPr>
+      <t>ľ</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="맑은 고딕"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>ad na produkt LG OLED evo AI</t>
+    </r>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>https://www.lg.com/sk/oled-tv</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t>Predný poh</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="238"/>
+      </rPr>
+      <t>ľ</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="맑은 고딕"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>ad na produkt LG OLED AI</t>
+    </r>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>https://www.lg.com/sk/qned-televizie</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t>Predný poh</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="238"/>
+      </rPr>
+      <t>ľ</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="맑은 고딕"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>ad na produkt LG QNED AI</t>
+    </r>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>https://www.lg.com/sk/nanocell-tv</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t>Predný poh</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="238"/>
+      </rPr>
+      <t>ľ</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="맑은 고딕"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>ad na produkt LG NanoCell AI</t>
+    </r>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t>Umelá inteligencia LG rozpozná vaše potreby a predloží riešenia, aby váš život plynul bez námahy pod</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="238"/>
+      </rPr>
+      <t>ľ</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="맑은 고딕"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>a vášho rytmu.</t>
+    </r>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t>Matka a syn spolo</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="238"/>
+      </rPr>
+      <t>č</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="맑은 고딕"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>ne používajú prá</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="238"/>
+      </rPr>
+      <t>č</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="맑은 고딕"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>ku LG s umelou inteligenciou a otá</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="238"/>
+      </rPr>
+      <t>č</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="맑은 고딕"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>aním ovláda</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="238"/>
+      </rPr>
+      <t>č</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="맑은 고딕"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>a aktivujú funkciu AI Wash. V tej istej sekvencii sa objaví muž, ktorý používa prenosný po</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="238"/>
+      </rPr>
+      <t>č</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="맑은 고딕"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>íta</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="238"/>
+      </rPr>
+      <t>č</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="맑은 고딕"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> LG gram.</t>
+    </r>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Pre váš bezstarostný život</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>https://www.lg.com/sk/chladnicky/lg-gmg960evee</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t>Predný poh</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="238"/>
+      </rPr>
+      <t>ľ</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="맑은 고딕"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>ad na produkt LG InstaView AI</t>
+    </r>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t>LG AI sa stará o vás, váš priestor a planétu, aby bol váš život spokojný, presne pod</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="238"/>
+      </rPr>
+      <t>ľ</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="맑은 고딕"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>a vašich predstáv.</t>
+    </r>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t>Do kancelárie vojde muž so psím vodítkom. Muž na sedadle vodi</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="238"/>
+      </rPr>
+      <t>č</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="맑은 고딕"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>a vyzerá smutne, ke</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="238"/>
+      </rPr>
+      <t>ď</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="맑은 고딕"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> mu LG AI ukazuje rodinnú fotografiu. Na displeji vozidla sa v detailnom zábere zobrazí, ako LG AI na</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="238"/>
+      </rPr>
+      <t>č</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="맑은 고딕"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>íta mapu a vráti sa k spomienke.</t>
+    </r>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Pre váš spokojný život</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>https://www.lg.com/cz/bytove-klimatizace/bytove-klimatizace</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t>Predný poh</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="238"/>
+      </rPr>
+      <t>ľ</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="맑은 고딕"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>ad na produkt LG DUALCOOL AI</t>
+    </r>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t>Bo</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="238"/>
+      </rPr>
+      <t>č</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="맑은 고딕"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>ný poh</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="238"/>
+      </rPr>
+      <t>ľ</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="맑은 고딕"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>ad na produkt ADAS vision</t>
+    </r>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t>Výber ponuky kávy s výzvou asistenta AI, interakcia používate</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="238"/>
+      </rPr>
+      <t>ľ</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="맑은 고딕"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>a s dotykovým rozhraním pohá</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="238"/>
+      </rPr>
+      <t>ň</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="맑은 고딕"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>aným multimodálnym riešením HMI s umelou inteligenciou</t>
+    </r>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t>Spotrebi</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="238"/>
+      </rPr>
+      <t>č</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="맑은 고딕"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>e</t>
+    </r>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Klimatizácie</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t>&lt;picture&gt;
+                        &lt;source srcset="./assets/image/ai-gate-image-product-category-tv-eyebrow-logo-desktop.svg" media="(min-width: 769px)"&gt;
+                        &lt;source srcset="./assets/image/ai-gate-image-product-category-tv-eyebrow-logo-mobile.svg" media="(max-width: 768px)"&gt;
+                        &lt;img src="./assets/image/ai-gate-image-product-category-tv-eyebrow-logo-mobile.svg" alt="LG AI TV" class="eyebrow-logo" loading="lazy"&gt;
+                      &lt;/picture&gt;
+                      Dokáže uspokoji</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="238"/>
+      </rPr>
+      <t>ť</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="맑은 고딕"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> všetky vaše potreby v oblasti zábavy</t>
+    </r>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t>LG AI TV sa u</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="238"/>
+      </rPr>
+      <t>č</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="맑은 고딕"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>í vaše divácke preferencie a chápe váš životný štýl, aby optimalizovala každý aspekt vášho televízneho zážitku a vytvorila ideálnu personalizovanú zábavu presne pre vás.</t>
+    </r>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t>Nad ovláda</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="238"/>
+      </rPr>
+      <t>č</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="맑은 고딕"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>om LG Magic Remote sa zobrazujú funkcie ako AI Voice ID, AI Search, AI Chatbot, AI Concierge, AI Picture Wizard a AI Sound Wizard.</t>
+    </r>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>https://www.lg.com/cz/tv-a-soundbars/ai-tv/</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t>Na obrazovke televízora LG OLED je domovská stránka systému webOS 25 plná aplikácií a zábavného obsahu. Pri televízore sa nachádza dia</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="238"/>
+      </rPr>
+      <t>ľ</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="맑은 고딕"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>kový ovláda</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="238"/>
+      </rPr>
+      <t>č</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="맑은 고딕"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> LG AI Magic Remote, ktorého tla</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="238"/>
+      </rPr>
+      <t>č</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="맑은 고딕"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>idlo AI je zvýraznené, akoby ho používate</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="238"/>
+      </rPr>
+      <t>ľ</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="맑은 고딕"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> aktivoval hlasom. Ved</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="238"/>
+      </rPr>
+      <t>ľ</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="맑은 고딕"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>a neho je re</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="238"/>
+      </rPr>
+      <t>č</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="맑은 고딕"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>ová bublina „“navrhni film, ktorý sa mi bude pá</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="238"/>
+      </rPr>
+      <t>č</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="맑은 고딕"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>i</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="238"/>
+      </rPr>
+      <t>ť</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="맑은 고딕"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>„“.</t>
+    </r>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t>Vyh</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="238"/>
+      </rPr>
+      <t>ľ</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="맑은 고딕"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>adávanie pomocou AI</t>
+    </r>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t>Obrazovka televízora LG OLED, ktorá ukazuje, ako funguje vyh</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="238"/>
+      </rPr>
+      <t>ľ</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="맑은 고딕"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>adávanie s umelou inteligenciou. Otvorí sa malé okno chatu, ktoré ukazuje, ako sa používate</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="238"/>
+      </rPr>
+      <t>ľ</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="맑은 고딕"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> pýtal na dostupné športové hry. Vyh</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="238"/>
+      </rPr>
+      <t>ľ</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="맑은 고딕"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>adávanie AI odpovedalo prostredníctvom chatu a zobrazením miniatúr rôzneho dostupného obsahu. K dispozícii je aj ponuka na položenie otázky Microsoft Copilot.</t>
+    </r>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t>Používanie dia</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="238"/>
+      </rPr>
+      <t>ľ</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="맑은 고딕"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>kového ovláda</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="238"/>
+      </rPr>
+      <t>č</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="맑은 고딕"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>a LG AI Magic Remote. Krátkym stla</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="238"/>
+      </rPr>
+      <t>č</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="맑은 고딕"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>ením tla</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="238"/>
+      </rPr>
+      <t>č</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="맑은 고딕"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>idla AI sa na obrazovke televízora OLED aktivuje asistent AI, ktorý potom navrhuje k</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="238"/>
+      </rPr>
+      <t>ľ</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="맑은 고딕"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>ú</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="238"/>
+      </rPr>
+      <t>č</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="맑은 고딕"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>ové slová.</t>
+    </r>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Na </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="238"/>
+      </rPr>
+      <t>ľ</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="맑은 고딕"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>avej strane obrazovky sa nachádza rozhranie Chatbot AI. Používate</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="238"/>
+      </rPr>
+      <t>ľ</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="맑은 고딕"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> oznámi chatbotovi, že obrazovka je príliš tmavá, a chatbot ponúkne riešenie požiadavky.</t>
+    </r>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Žena spievajúca do mikrofónu so slúchadlami, zvýraznená vylepšením zvuku procesorom LG α11 AI</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t>Dia</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="238"/>
+      </rPr>
+      <t>ľ</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="맑은 고딕"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>kový ovláda</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="238"/>
+      </rPr>
+      <t>č</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="맑은 고딕"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> AI Magic</t>
+    </r>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t>Dve prepojené scény s ovláda</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="238"/>
+      </rPr>
+      <t>č</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="맑은 고딕"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>om LG AI Magic Remote pred televízorom - prvá zobrazuje sci-fi scénu, druhá zobrazuje domovskú obrazovku s personalizovaným obsahom</t>
+    </r>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t>*Funkcie umelej inteligencie LG využívajú vyškolené algoritmy založené na hlbokom u</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="238"/>
+      </rPr>
+      <t>č</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="맑은 고딕"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">ení na zvýšenie rozlíšenia obrazu a zmiešavanie zvuku v reálnom </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="238"/>
+      </rPr>
+      <t>č</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="맑은 고딕"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>ase.</t>
+    </r>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>**Všetky televízory LG so systémom webOS 24 sú vybavené funkciou AI Customization, okrem televízorov bez svetelných senzorov.</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t>&lt;picture&gt;
+                        &lt;source srcset="./assets/image/ai-gate-image-product-category-audio-eyebrow-logo-desktop.svg" media="(min-width: 769px)"&gt;
+                        &lt;source srcset="./assets/image/ai-gate-image-product-category-audio-eyebrow-logo-mobile.svg" media="(max-width: 768px)"&gt;
+                        &lt;img src="./assets/image/ai-gate-image-product-category-audio-eyebrow-logo-mobile.svg" alt="LG AI Audio" class="eyebrow-logo" loading="lazy"&gt;
+                      &lt;/picture&gt;
+                      Znie to jedine</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="238"/>
+      </rPr>
+      <t>č</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="맑은 고딕"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>ne</t>
+    </r>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t>LG xboom AI analyzuje a upravuje zvuk tak, aby vyhovoval žánru a priestoru. V</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="238"/>
+      </rPr>
+      <t>ď</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="맑은 고딕"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>aka osvetleniu AI, ktoré zlepšuje atmosféru a harmonizuje s hudbou, si môžete vychutna</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="238"/>
+      </rPr>
+      <t>ť</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="맑은 고딕"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> zvuk a atmosféru unikátne a správne.</t>
+    </r>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Užite si nový zvukový zážitok s technológiou &lt;br&gt;
+                          LG xboom AI</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>https://www.lg.com/sk/audio-systemy</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t>Žena a muž sa objímajú v obýva</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="238"/>
+      </rPr>
+      <t>č</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="맑은 고딕"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>ke a ved</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="238"/>
+      </rPr>
+      <t>ľ</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="맑은 고딕"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>a nich je zapnutý reproduktor XBOOM.</t>
+    </r>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Reproduktor LG XBOOM s režimami zvuku AI vrátane Bass Boost, Voice Enhance a Standard</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>AI zvuk</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>AI osvetlenie</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Reproduktor LG XBOOM s osvetlením AI, ktoré sa prispôsobuje hlasovým, ambientným a párty režimom</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Reproduktor LG XBOOM umiestnený na stole v </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="238"/>
+      </rPr>
+      <t>č</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="맑은 고딕"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>ervenej miestnosti so stenami s mriežkovým vzorom a moderným nábytkom</t>
+    </r>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>AI kalibrácia</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Technológia LG WashTower AI rozpoznáva, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="238"/>
+      </rPr>
+      <t>č</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="맑은 고딕"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>o periete, a poskytuje optimalizované pranie pre citlivú starostlivos</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="238"/>
+      </rPr>
+      <t>ť</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="맑은 고딕"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> o tkaniny, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="238"/>
+      </rPr>
+      <t>č</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="맑은 고딕"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>ím zakaždým zaistí dokonalé vypranie každej náplne.</t>
+    </r>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t>&lt;picture&gt;
+                        &lt;source srcset="./assets/image/ai-gate-image-product-category-appliances-eyebrow-logo-desktop.svg" media="(min-width: 769px)"&gt;
+                        &lt;source srcset="./assets/image/ai-gate-image-product-category-appliances-eyebrow-logo-mobile.svg" media="(max-width: 768px)"&gt;
+                        &lt;img src="./assets/image/ai-gate-image-product-category-appliances-eyebrow-logo-mobile.svg" alt="Spotrebi</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="238"/>
+      </rPr>
+      <t>č</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="맑은 고딕"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>e" class="eyebrow-logo" loading="lazy"&gt;
+                      &lt;/picture&gt;
+                      Z</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="238"/>
+      </rPr>
+      <t>ľ</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="맑은 고딕"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>ah</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="238"/>
+      </rPr>
+      <t>č</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="맑은 고딕"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>ite si každú zá</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="238"/>
+      </rPr>
+      <t>ť</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="맑은 고딕"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>až</t>
+    </r>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>https://www.lg.com/sk/pracky/lg-wt1210wwf</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t>Vstavaná prá</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="238"/>
+      </rPr>
+      <t>č</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="맑은 고딕"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>ka a suši</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="238"/>
+      </rPr>
+      <t>č</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="맑은 고딕"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>ka LG v modernej prá</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="238"/>
+      </rPr>
+      <t>č</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="맑은 고딕"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>ovni s drevenými skri</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="238"/>
+      </rPr>
+      <t>ň</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="맑은 고딕"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>ami a lavicami na sedenie</t>
+    </r>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t>Ru</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="238"/>
+      </rPr>
+      <t>č</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="맑은 고딕"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>né nastavenie cyklu AI Wash na prá</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="238"/>
+      </rPr>
+      <t>č</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="맑은 고딕"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>ke LG pomocou inteligentného voli</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="238"/>
+      </rPr>
+      <t>č</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="맑은 고딕"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>a</t>
+    </r>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t>Výber cyklu AI Dry na suši</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="238"/>
+      </rPr>
+      <t>č</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="맑은 고딕"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>ke LG pomocou digitálneho ovládacieho voli</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="238"/>
+      </rPr>
+      <t>č</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="맑은 고딕"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>a</t>
+    </r>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>AI pranie</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>AI sušenie</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t>*Tento produkt sa bude vo vybraných krajinách uvo</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="238"/>
+      </rPr>
+      <t>ľň</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="맑은 고딕"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>ova</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="238"/>
+      </rPr>
+      <t>ť</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="맑은 고딕"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> postupne.</t>
+    </r>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t>**Snímanie pomocou systému AI sa aktivuje, ke</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="238"/>
+      </rPr>
+      <t>ď</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="맑은 고딕"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> je hmotnos</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="238"/>
+      </rPr>
+      <t>ť</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="맑은 고딕"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> nákplne nižšia ako 6 kg.</t>
+    </r>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t>***AI Wash by sa malo používa</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="238"/>
+      </rPr>
+      <t>ť</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="맑은 고딕"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> len s podobnými typmi tkanín [nie všetky tkaniny sú rozpoznané] a vhodným pracím prostriedkom.</t>
+    </r>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>&lt;picture&gt;
+                        &lt;source srcset="./assets/image/ai-gate-image-product-category-air-conditioning-eyebrow-logo-desktop.svg" media="(min-width: 769px)"&gt;
+                        &lt;source srcset="./assets/image/ai-gate-image-product-category-air-conditioning-eyebrow-logo-mobile.svg" media="(max-width: 768px)"&gt;
+                        &lt;img src="./assets/image/ai-gate-image-product-category-air-conditioning-eyebrow-logo-mobile.svg" alt="Klimatizácie" class="eyebrow-logo" loading="lazy"&gt;
+                      &lt;/picture&gt;
+                      Pohodlie s dokonale vyladeným chladením</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t>LG DUALCOOL AI sa stará o optimálnu klímu, udržiava pohodlie a zárove</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="238"/>
+      </rPr>
+      <t>ň</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="맑은 고딕"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> optimalizuje energetickú ú</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="238"/>
+      </rPr>
+      <t>č</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="맑은 고딕"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>innos</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="238"/>
+      </rPr>
+      <t>ť</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="맑은 고딕"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="238"/>
+      </rPr>
+      <t>č</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="맑은 고딕"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>ím pomáha šetri</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="238"/>
+      </rPr>
+      <t>ť</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="맑은 고딕"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> náklady. S LG AI Air zažijete dokonale prispôsobené chladenie pre vaše pohodlie.</t>
+    </r>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Pomocou technológie ThinQ AI, klimatizácia LG DUAL Inverter chladí modernú obývaciu izbu, v ktorej na pohovke sedí žena.</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Zažite optimalizovaný dizajn s technológiou &lt;br&gt;
+                          LG AI Air</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t>Žena relaxuje v inteligentnej obýva</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="238"/>
+      </rPr>
+      <t>č</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="맑은 고딕"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>ke, zatia</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="238"/>
+      </rPr>
+      <t>ľ</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="맑은 고딕"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="238"/>
+      </rPr>
+      <t>č</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="맑은 고딕"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>o klimatizácia LG AI automaticky upravuje teplotu, prúdenie vzduchu a vlhkos</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="238"/>
+      </rPr>
+      <t>ť</t>
+    </r>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Rozhranie smartfónu zobrazujúce graf spotreby energie pred klimatizáciou LG, zvýraznenie AI kW Manager na efektívne monitorovanie energie</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Manažér AI kW</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t>*Air AI sa dá ovláda</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="238"/>
+      </rPr>
+      <t>ť</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="맑은 고딕"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> pomocou dia</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="238"/>
+      </rPr>
+      <t>ľ</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="맑은 고딕"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>kového ovládania a ThinQ.</t>
+    </r>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>**AI Air je k dispozícii v režime chladenia aj vykurovania.</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t>***Po</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="238"/>
+      </rPr>
+      <t>č</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="맑은 고딕"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>as používania AI Air sa objem vzduchu a smer prúdenia vzduchu automaticky upravujú pod</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="238"/>
+      </rPr>
+      <t>ľ</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="맑은 고딕"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>a situácie a AI Air sa vypne, ke</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="238"/>
+      </rPr>
+      <t>ď</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="맑은 고딕"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> sa zmení smer prúdenia vzduchu.</t>
+    </r>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t>****Pri aktivácii funkcie AI Air radarový sníma</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="238"/>
+      </rPr>
+      <t>č</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="맑은 고딕"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> zistí polohu používate</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="238"/>
+      </rPr>
+      <t>ľ</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="맑은 고딕"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>a a automaticky aktivuje priamy/nepriamy smer  prúdenia vzduchu.</t>
+    </r>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t>*****Vzdialenos</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="238"/>
+      </rPr>
+      <t>ť</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="맑은 고딕"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> snímania radarového sníma</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="238"/>
+      </rPr>
+      <t>č</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="맑은 고딕"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>a je do 5 m, pri</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="238"/>
+      </rPr>
+      <t>č</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="맑은 고딕"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>om v závislosti od prostredia inštalácie a používania výrobku môžu by</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="238"/>
+      </rPr>
+      <t>ť</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="맑은 고딕"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> rozdiely vo vzdialenosti snímania.</t>
+    </r>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t>******Táto funkcia funguje len s modelmi, ktoré majú radarové sníma</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="238"/>
+      </rPr>
+      <t>č</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="맑은 고딕"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>e.</t>
+    </r>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t>ThinQ® pomáha prinies</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="238"/>
+      </rPr>
+      <t>ť</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="맑은 고딕"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> život do reality</t>
+    </r>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t>Platforma pre inteligentné spotrebi</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="238"/>
+      </rPr>
+      <t>č</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="맑은 고딕"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>e a zariadenia LG ThinQ vám umožní ovláda</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="238"/>
+      </rPr>
+      <t>ť</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="맑은 고딕"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> a využíva</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="238"/>
+      </rPr>
+      <t>ť</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="맑은 고딕"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> pohodlie na dosah ruky, aby vám pomohla zjednoduši</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="238"/>
+      </rPr>
+      <t>ť</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="맑은 고딕"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> život a užíva</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="238"/>
+      </rPr>
+      <t>ť</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="맑은 고딕"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> si pohodlie domova.</t>
+    </r>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>https://www.lg.com/sk/domace-spotrebice/thinq</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="238"/>
+      </rPr>
+      <t>Č</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="맑은 고딕"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>lovek drží smartfón s otvorenou aplikáciou LG ThinQ a po</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="238"/>
+      </rPr>
+      <t>č</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="맑은 고딕"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>as pitia kávy spravuje inteligentné domáce zariadenia.</t>
+    </r>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t>V modernej inteligentnej kuchyni žena pomocou hlasového príkazu spúš</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="238"/>
+      </rPr>
+      <t>ť</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="맑은 고딕"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>a prá</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="238"/>
+      </rPr>
+      <t>č</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="맑은 고딕"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>ku s umelou inteligenciou LG ThinQ, zatia</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="238"/>
+      </rPr>
+      <t>ľ</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="맑은 고딕"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="238"/>
+      </rPr>
+      <t>č</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="맑은 고딕"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">o muž v úzadí na pohovke </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="238"/>
+      </rPr>
+      <t>č</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="맑은 고딕"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>íta.</t>
+    </r>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Jednoduché ovládanie s hlasovým asistentom</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Povedzte zariadeniu LG, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="238"/>
+      </rPr>
+      <t>č</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="맑은 고딕"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>o presne potrebujete, a reproduktor s umelou inteligenciou si vás vypo</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="238"/>
+      </rPr>
+      <t>č</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="맑은 고딕"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>uje a skontroluje priebeh cyklu a dá vám to na vedomie.</t>
+    </r>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t>a displeji smartfónu sa zobrazuje aplikácia LG ThinQ, ktorá ovláda vstavanú rúru LG InstaView Slide-In Range a umož</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="238"/>
+      </rPr>
+      <t>ň</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="맑은 고딕"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>uje efektívnu údržbu výrobku v kuchyni.</t>
+    </r>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Efektívna údržba produktov</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t>Prostredníctvom aplikácie LG ThinQ môžete kontrolova</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="238"/>
+      </rPr>
+      <t>ť</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="맑은 고딕"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> svoj spotrebi</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="238"/>
+      </rPr>
+      <t>č</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="맑은 고딕"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> LG, s</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="238"/>
+      </rPr>
+      <t>ť</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="맑은 고딕"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>ahova</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="238"/>
+      </rPr>
+      <t>ť</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="맑은 고딕"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> nové cykly, sledova</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="238"/>
+      </rPr>
+      <t>ť</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="맑은 고딕"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> priebeh cyklu a mnoho </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="238"/>
+      </rPr>
+      <t>ď</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="맑은 고딕"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>alšieho.</t>
+    </r>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Viac o LG Láskavá inteligencia</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t>Spolo</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="238"/>
+      </rPr>
+      <t>č</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="맑은 고딕"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>nos</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="238"/>
+      </rPr>
+      <t>ť</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="맑은 고딕"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> LG posil</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="238"/>
+      </rPr>
+      <t>ň</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="맑은 고딕"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>uje vedúce postavenie v oblasti kybernetickej bezpe</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="238"/>
+      </rPr>
+      <t>č</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="맑은 고딕"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>nosti v</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="238"/>
+      </rPr>
+      <t>ď</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="맑은 고딕"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>aka akreditácii KOLAS na testovanie kybernetickej bezpe</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="238"/>
+      </rPr>
+      <t>č</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="맑은 고딕"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>nosti IoT</t>
+    </r>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t>Riadiaci pracovník spolo</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="238"/>
+      </rPr>
+      <t>č</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="맑은 고딕"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>nosti LG Electronics s certifikátom o akreditácii pre kybernetickú bezpe</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="238"/>
+      </rPr>
+      <t>č</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="맑은 고딕"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>nos</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="238"/>
+      </rPr>
+      <t>ť</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="맑은 고딕"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>, v pozadí grafika digitálnej bezpe</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="238"/>
+      </rPr>
+      <t>č</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="맑은 고딕"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>nosti</t>
+    </r>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Návštevníci si na výstave technológií obzerajú zakrivený LED displej LG so sloganom "Life's Good 24/7</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t>V spolo</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="238"/>
+      </rPr>
+      <t>č</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="맑은 고딕"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>nosti LG sme si kládli otázku: Pre</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="238"/>
+      </rPr>
+      <t>č</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="맑은 고딕"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>o by mala umelá inteligencia existova</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="238"/>
+      </rPr>
+      <t>ť</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="맑은 고딕"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>? &lt;br&gt;
+              Po dlhom uvažovaní sme našli odpove</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="238"/>
+      </rPr>
+      <t>ď</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="맑은 고딕"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>. &lt;br&gt;&lt;br&gt;
+              Pre nás AI presahuje rámec umelej inteligencie - je to láskavá inteligencia. &lt;br&gt;&lt;br&gt;
+              As AI becomes a part of our daily lives, &lt;br&gt;
+              by mala pomôc</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="238"/>
+      </rPr>
+      <t>ť</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="맑은 고딕"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> vytvori</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="238"/>
+      </rPr>
+      <t>ť</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="맑은 고딕"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> lepší život, ktorý si všetci zaslúžime. &lt;br&gt;&lt;br&gt;
+              Preto LG AI za</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="238"/>
+      </rPr>
+      <t>č</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="맑은 고딕"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">ína s Vami láskyplne prostredníctvom &lt;br&gt;
+              vnímania a porozumenia, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="238"/>
+      </rPr>
+      <t>ď</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="맑은 고딕"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>alej sa stará o Váš život.
+              &lt;strong&gt;Zistite, ako je Life's Good s umelou inteligenciou LG&lt;/strong&gt;</t>
+    </r>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Zoznámte sa s novou generáciou &lt;br&gt;
+                          LG AI TV</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Objavte nový spôsob života s technológiou &lt;br&gt;
+                           LG AI Core Tech</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t>****AI Dry je k dispozícii len pre nápl</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="238"/>
+      </rPr>
+      <t>ň</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="맑은 고딕"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> s hmotnos</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="238"/>
+      </rPr>
+      <t>ť</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="맑은 고딕"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>ou pod 5 kg a s tkaninami s rovnakou úrov</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="238"/>
+      </rPr>
+      <t>ň</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="맑은 고딕"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>ou nasiakavosti.</t>
+    </r>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="6">
+  <fonts count="8">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -24037,6 +27652,21 @@
       <charset val="178"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="238"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="맑은 고딕"/>
+      <family val="2"/>
+      <charset val="238"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="3">
     <fill>
@@ -24064,7 +27694,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -24076,6 +27706,7 @@
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="표준" xfId="0" builtinId="0"/>
@@ -30717,4 +34348,1276 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BB88BCCA-2AF6-E44E-B910-B08F30094E46}">
+  <dimension ref="A1:B166"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="17"/>
+  <cols>
+    <col min="1" max="1" width="15" customWidth="1"/>
+    <col min="2" max="2" width="120" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" s="1" customFormat="1">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" ht="198">
+      <c r="A2" t="s">
+        <v>2</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>476</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2">
+      <c r="A3" t="s">
+        <v>4</v>
+      </c>
+      <c r="B3" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2">
+      <c r="A4" t="s">
+        <v>313</v>
+      </c>
+      <c r="B4" t="s">
+        <v>477</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" ht="144">
+      <c r="A5" t="s">
+        <v>2</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>571</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2">
+      <c r="A6" t="s">
+        <v>4</v>
+      </c>
+      <c r="B6" t="s">
+        <v>478</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2">
+      <c r="A7" t="s">
+        <v>2</v>
+      </c>
+      <c r="B7" t="s">
+        <v>479</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2">
+      <c r="A8" t="s">
+        <v>2</v>
+      </c>
+      <c r="B8" t="s">
+        <v>480</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2">
+      <c r="A9" t="s">
+        <v>2</v>
+      </c>
+      <c r="B9" t="s">
+        <v>481</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2">
+      <c r="A10" t="s">
+        <v>2</v>
+      </c>
+      <c r="B10" t="s">
+        <v>482</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" ht="36">
+      <c r="A11" t="s">
+        <v>2</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>483</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2">
+      <c r="A12" t="s">
+        <v>2</v>
+      </c>
+      <c r="B12" t="s">
+        <v>485</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2">
+      <c r="A13" t="s">
+        <v>13</v>
+      </c>
+      <c r="B13" s="3" t="s">
+        <v>486</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2">
+      <c r="A14" t="s">
+        <v>4</v>
+      </c>
+      <c r="B14" t="s">
+        <v>487</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2">
+      <c r="A15" t="s">
+        <v>2</v>
+      </c>
+      <c r="B15" t="s">
+        <v>484</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2">
+      <c r="A16" t="s">
+        <v>13</v>
+      </c>
+      <c r="B16" s="3" t="s">
+        <v>488</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2">
+      <c r="A17" t="s">
+        <v>4</v>
+      </c>
+      <c r="B17" t="s">
+        <v>489</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2">
+      <c r="A18" t="s">
+        <v>2</v>
+      </c>
+      <c r="B18" t="s">
+        <v>484</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2">
+      <c r="A19" t="s">
+        <v>13</v>
+      </c>
+      <c r="B19" s="3" t="s">
+        <v>490</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2">
+      <c r="A20" t="s">
+        <v>4</v>
+      </c>
+      <c r="B20" t="s">
+        <v>491</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2">
+      <c r="A21" t="s">
+        <v>2</v>
+      </c>
+      <c r="B21" t="s">
+        <v>484</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2">
+      <c r="A22" t="s">
+        <v>13</v>
+      </c>
+      <c r="B22" s="3" t="s">
+        <v>492</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2">
+      <c r="A23" t="s">
+        <v>4</v>
+      </c>
+      <c r="B23" t="s">
+        <v>493</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2">
+      <c r="A24" t="s">
+        <v>2</v>
+      </c>
+      <c r="B24" t="s">
+        <v>484</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2">
+      <c r="A25" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="26" spans="1:2">
+      <c r="A26" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="27" spans="1:2">
+      <c r="A27" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="28" spans="1:2">
+      <c r="A28" t="s">
+        <v>2</v>
+      </c>
+      <c r="B28" t="s">
+        <v>494</v>
+      </c>
+    </row>
+    <row r="29" spans="1:2">
+      <c r="A29" t="s">
+        <v>2</v>
+      </c>
+      <c r="B29" t="s">
+        <v>495</v>
+      </c>
+    </row>
+    <row r="30" spans="1:2">
+      <c r="A30" t="s">
+        <v>2</v>
+      </c>
+      <c r="B30" t="s">
+        <v>496</v>
+      </c>
+    </row>
+    <row r="31" spans="1:2">
+      <c r="A31" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="32" spans="1:2">
+      <c r="A32" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="33" spans="1:2">
+      <c r="A33" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="34" spans="1:2">
+      <c r="A34" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="35" spans="1:2">
+      <c r="A35" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="36" spans="1:2">
+      <c r="A36" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="37" spans="1:2">
+      <c r="A37" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="38" spans="1:2">
+      <c r="A38" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="39" spans="1:2">
+      <c r="A39" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="40" spans="1:2">
+      <c r="A40" t="s">
+        <v>13</v>
+      </c>
+      <c r="B40" s="3" t="s">
+        <v>497</v>
+      </c>
+    </row>
+    <row r="41" spans="1:2">
+      <c r="A41" t="s">
+        <v>4</v>
+      </c>
+      <c r="B41" t="s">
+        <v>498</v>
+      </c>
+    </row>
+    <row r="42" spans="1:2">
+      <c r="A42" t="s">
+        <v>2</v>
+      </c>
+      <c r="B42" t="s">
+        <v>484</v>
+      </c>
+    </row>
+    <row r="43" spans="1:2">
+      <c r="A43" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="44" spans="1:2">
+      <c r="A44" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="45" spans="1:2">
+      <c r="A45" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="46" spans="1:2">
+      <c r="A46" t="s">
+        <v>2</v>
+      </c>
+      <c r="B46" t="s">
+        <v>499</v>
+      </c>
+    </row>
+    <row r="47" spans="1:2">
+      <c r="A47" t="s">
+        <v>2</v>
+      </c>
+      <c r="B47" t="s">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="48" spans="1:2">
+      <c r="A48" t="s">
+        <v>2</v>
+      </c>
+      <c r="B48" t="s">
+        <v>501</v>
+      </c>
+    </row>
+    <row r="49" spans="1:2">
+      <c r="A49" t="s">
+        <v>13</v>
+      </c>
+      <c r="B49" s="3" t="s">
+        <v>502</v>
+      </c>
+    </row>
+    <row r="50" spans="1:2">
+      <c r="A50" t="s">
+        <v>4</v>
+      </c>
+      <c r="B50" t="s">
+        <v>503</v>
+      </c>
+    </row>
+    <row r="51" spans="1:2">
+      <c r="A51" t="s">
+        <v>2</v>
+      </c>
+      <c r="B51" t="s">
+        <v>484</v>
+      </c>
+    </row>
+    <row r="52" spans="1:2">
+      <c r="A52" t="s">
+        <v>13</v>
+      </c>
+      <c r="B52" s="3" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="53" spans="1:2">
+      <c r="A53" t="s">
+        <v>4</v>
+      </c>
+      <c r="B53" t="s">
+        <v>504</v>
+      </c>
+    </row>
+    <row r="54" spans="1:2">
+      <c r="A54" t="s">
+        <v>2</v>
+      </c>
+      <c r="B54" t="s">
+        <v>484</v>
+      </c>
+    </row>
+    <row r="55" spans="1:2">
+      <c r="A55" t="s">
+        <v>13</v>
+      </c>
+      <c r="B55" s="3" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="56" spans="1:2">
+      <c r="A56" t="s">
+        <v>4</v>
+      </c>
+      <c r="B56" t="s">
+        <v>505</v>
+      </c>
+    </row>
+    <row r="57" spans="1:2">
+      <c r="A57" t="s">
+        <v>2</v>
+      </c>
+      <c r="B57" t="s">
+        <v>484</v>
+      </c>
+    </row>
+    <row r="58" spans="1:2">
+      <c r="A58" t="s">
+        <v>2</v>
+      </c>
+      <c r="B58" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="59" spans="1:2">
+      <c r="A59" t="s">
+        <v>2</v>
+      </c>
+      <c r="B59" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="60" spans="1:2">
+      <c r="A60" t="s">
+        <v>2</v>
+      </c>
+      <c r="B60" t="s">
+        <v>506</v>
+      </c>
+    </row>
+    <row r="61" spans="1:2">
+      <c r="A61" t="s">
+        <v>2</v>
+      </c>
+      <c r="B61" t="s">
+        <v>507</v>
+      </c>
+    </row>
+    <row r="62" spans="1:2">
+      <c r="A62" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="63" spans="1:2" ht="162">
+      <c r="A63" t="s">
+        <v>2</v>
+      </c>
+      <c r="B63" s="2" t="s">
+        <v>508</v>
+      </c>
+    </row>
+    <row r="64" spans="1:2">
+      <c r="A64" t="s">
+        <v>4</v>
+      </c>
+      <c r="B64" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="65" spans="1:2">
+      <c r="A65" t="s">
+        <v>2</v>
+      </c>
+      <c r="B65" t="s">
+        <v>509</v>
+      </c>
+    </row>
+    <row r="66" spans="1:2">
+      <c r="A66" t="s">
+        <v>4</v>
+      </c>
+      <c r="B66" t="s">
+        <v>510</v>
+      </c>
+    </row>
+    <row r="67" spans="1:2" ht="36">
+      <c r="A67" t="s">
+        <v>2</v>
+      </c>
+      <c r="B67" s="2" t="s">
+        <v>572</v>
+      </c>
+    </row>
+    <row r="68" spans="1:2">
+      <c r="A68" t="s">
+        <v>2</v>
+      </c>
+      <c r="B68" t="s">
+        <v>484</v>
+      </c>
+    </row>
+    <row r="69" spans="1:2">
+      <c r="A69" t="s">
+        <v>13</v>
+      </c>
+      <c r="B69" s="3" t="s">
+        <v>511</v>
+      </c>
+    </row>
+    <row r="70" spans="1:2">
+      <c r="A70" t="s">
+        <v>4</v>
+      </c>
+      <c r="B70" t="s">
+        <v>512</v>
+      </c>
+    </row>
+    <row r="71" spans="1:2">
+      <c r="A71" t="s">
+        <v>2</v>
+      </c>
+      <c r="B71" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="72" spans="1:2">
+      <c r="A72" t="s">
+        <v>4</v>
+      </c>
+      <c r="B72" t="s">
+        <v>514</v>
+      </c>
+    </row>
+    <row r="73" spans="1:2">
+      <c r="A73" t="s">
+        <v>2</v>
+      </c>
+      <c r="B73" t="s">
+        <v>513</v>
+      </c>
+    </row>
+    <row r="74" spans="1:2">
+      <c r="A74" t="s">
+        <v>4</v>
+      </c>
+      <c r="B74" t="s">
+        <v>515</v>
+      </c>
+    </row>
+    <row r="75" spans="1:2">
+      <c r="A75" t="s">
+        <v>2</v>
+      </c>
+      <c r="B75" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="76" spans="1:2">
+      <c r="A76" t="s">
+        <v>4</v>
+      </c>
+      <c r="B76" t="s">
+        <v>516</v>
+      </c>
+    </row>
+    <row r="77" spans="1:2">
+      <c r="A77" t="s">
+        <v>2</v>
+      </c>
+      <c r="B77" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="78" spans="1:2">
+      <c r="A78" t="s">
+        <v>4</v>
+      </c>
+      <c r="B78" t="s">
+        <v>517</v>
+      </c>
+    </row>
+    <row r="79" spans="1:2">
+      <c r="A79" t="s">
+        <v>2</v>
+      </c>
+      <c r="B79" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="80" spans="1:2">
+      <c r="A80" t="s">
+        <v>4</v>
+      </c>
+      <c r="B80" t="s">
+        <v>519</v>
+      </c>
+    </row>
+    <row r="81" spans="1:2">
+      <c r="A81" t="s">
+        <v>2</v>
+      </c>
+      <c r="B81" t="s">
+        <v>518</v>
+      </c>
+    </row>
+    <row r="82" spans="1:2">
+      <c r="A82" t="s">
+        <v>2</v>
+      </c>
+      <c r="B82" t="s">
+        <v>520</v>
+      </c>
+    </row>
+    <row r="83" spans="1:2">
+      <c r="A83" t="s">
+        <v>2</v>
+      </c>
+      <c r="B83" t="s">
+        <v>521</v>
+      </c>
+    </row>
+    <row r="84" spans="1:2" ht="162">
+      <c r="A84" t="s">
+        <v>2</v>
+      </c>
+      <c r="B84" s="2" t="s">
+        <v>522</v>
+      </c>
+    </row>
+    <row r="85" spans="1:2">
+      <c r="A85" t="s">
+        <v>4</v>
+      </c>
+      <c r="B85" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="86" spans="1:2">
+      <c r="A86" t="s">
+        <v>2</v>
+      </c>
+      <c r="B86" t="s">
+        <v>523</v>
+      </c>
+    </row>
+    <row r="87" spans="1:2">
+      <c r="A87" t="s">
+        <v>4</v>
+      </c>
+      <c r="B87" t="s">
+        <v>526</v>
+      </c>
+    </row>
+    <row r="88" spans="1:2" ht="36">
+      <c r="A88" t="s">
+        <v>2</v>
+      </c>
+      <c r="B88" s="2" t="s">
+        <v>524</v>
+      </c>
+    </row>
+    <row r="89" spans="1:2">
+      <c r="A89" t="s">
+        <v>2</v>
+      </c>
+      <c r="B89" t="s">
+        <v>484</v>
+      </c>
+    </row>
+    <row r="90" spans="1:2">
+      <c r="A90" t="s">
+        <v>13</v>
+      </c>
+      <c r="B90" s="3" t="s">
+        <v>525</v>
+      </c>
+    </row>
+    <row r="91" spans="1:2">
+      <c r="A91" t="s">
+        <v>4</v>
+      </c>
+      <c r="B91" t="s">
+        <v>527</v>
+      </c>
+    </row>
+    <row r="92" spans="1:2">
+      <c r="A92" t="s">
+        <v>2</v>
+      </c>
+      <c r="B92" t="s">
+        <v>528</v>
+      </c>
+    </row>
+    <row r="93" spans="1:2">
+      <c r="A93" t="s">
+        <v>4</v>
+      </c>
+      <c r="B93" t="s">
+        <v>530</v>
+      </c>
+    </row>
+    <row r="94" spans="1:2">
+      <c r="A94" t="s">
+        <v>2</v>
+      </c>
+      <c r="B94" t="s">
+        <v>529</v>
+      </c>
+    </row>
+    <row r="95" spans="1:2">
+      <c r="A95" t="s">
+        <v>4</v>
+      </c>
+      <c r="B95" t="s">
+        <v>531</v>
+      </c>
+    </row>
+    <row r="96" spans="1:2">
+      <c r="A96" t="s">
+        <v>2</v>
+      </c>
+      <c r="B96" t="s">
+        <v>532</v>
+      </c>
+    </row>
+    <row r="97" spans="1:2">
+      <c r="A97" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="98" spans="1:2" ht="162">
+      <c r="A98" t="s">
+        <v>2</v>
+      </c>
+      <c r="B98" s="2" t="s">
+        <v>534</v>
+      </c>
+    </row>
+    <row r="99" spans="1:2">
+      <c r="A99" t="s">
+        <v>4</v>
+      </c>
+      <c r="B99" t="s">
+        <v>506</v>
+      </c>
+    </row>
+    <row r="100" spans="1:2">
+      <c r="A100" t="s">
+        <v>2</v>
+      </c>
+      <c r="B100" t="s">
+        <v>533</v>
+      </c>
+    </row>
+    <row r="101" spans="1:2">
+      <c r="A101" t="s">
+        <v>4</v>
+      </c>
+      <c r="B101" t="s">
+        <v>536</v>
+      </c>
+    </row>
+    <row r="102" spans="1:2" ht="36">
+      <c r="A102" t="s">
+        <v>2</v>
+      </c>
+      <c r="B102" s="2" t="s">
+        <v>573</v>
+      </c>
+    </row>
+    <row r="103" spans="1:2">
+      <c r="A103" t="s">
+        <v>2</v>
+      </c>
+      <c r="B103" t="s">
+        <v>484</v>
+      </c>
+    </row>
+    <row r="104" spans="1:2">
+      <c r="A104" t="s">
+        <v>13</v>
+      </c>
+      <c r="B104" s="3" t="s">
+        <v>535</v>
+      </c>
+    </row>
+    <row r="105" spans="1:2">
+      <c r="A105" t="s">
+        <v>4</v>
+      </c>
+      <c r="B105" t="s">
+        <v>537</v>
+      </c>
+    </row>
+    <row r="106" spans="1:2">
+      <c r="A106" t="s">
+        <v>2</v>
+      </c>
+      <c r="B106" t="s">
+        <v>539</v>
+      </c>
+    </row>
+    <row r="107" spans="1:2">
+      <c r="A107" t="s">
+        <v>4</v>
+      </c>
+      <c r="B107" t="s">
+        <v>538</v>
+      </c>
+    </row>
+    <row r="108" spans="1:2">
+      <c r="A108" t="s">
+        <v>2</v>
+      </c>
+      <c r="B108" t="s">
+        <v>540</v>
+      </c>
+    </row>
+    <row r="109" spans="1:2">
+      <c r="A109" t="s">
+        <v>2</v>
+      </c>
+      <c r="B109" t="s">
+        <v>541</v>
+      </c>
+    </row>
+    <row r="110" spans="1:2">
+      <c r="A110" t="s">
+        <v>2</v>
+      </c>
+      <c r="B110" t="s">
+        <v>542</v>
+      </c>
+    </row>
+    <row r="111" spans="1:2">
+      <c r="A111" t="s">
+        <v>2</v>
+      </c>
+      <c r="B111" t="s">
+        <v>543</v>
+      </c>
+    </row>
+    <row r="112" spans="1:2">
+      <c r="A112" t="s">
+        <v>2</v>
+      </c>
+      <c r="B112" t="s">
+        <v>574</v>
+      </c>
+    </row>
+    <row r="113" spans="1:2" ht="162">
+      <c r="A113" t="s">
+        <v>2</v>
+      </c>
+      <c r="B113" s="2" t="s">
+        <v>544</v>
+      </c>
+    </row>
+    <row r="114" spans="1:2">
+      <c r="A114" t="s">
+        <v>4</v>
+      </c>
+      <c r="B114" t="s">
+        <v>507</v>
+      </c>
+    </row>
+    <row r="115" spans="1:2">
+      <c r="A115" t="s">
+        <v>2</v>
+      </c>
+      <c r="B115" t="s">
+        <v>545</v>
+      </c>
+    </row>
+    <row r="116" spans="1:2">
+      <c r="A116" t="s">
+        <v>4</v>
+      </c>
+      <c r="B116" t="s">
+        <v>546</v>
+      </c>
+    </row>
+    <row r="117" spans="1:2" ht="36">
+      <c r="A117" t="s">
+        <v>2</v>
+      </c>
+      <c r="B117" s="2" t="s">
+        <v>547</v>
+      </c>
+    </row>
+    <row r="118" spans="1:2">
+      <c r="A118" t="s">
+        <v>2</v>
+      </c>
+      <c r="B118" t="s">
+        <v>484</v>
+      </c>
+    </row>
+    <row r="119" spans="1:2">
+      <c r="A119" t="s">
+        <v>13</v>
+      </c>
+      <c r="B119" s="3" t="s">
+        <v>502</v>
+      </c>
+    </row>
+    <row r="120" spans="1:2">
+      <c r="A120" t="s">
+        <v>4</v>
+      </c>
+      <c r="B120" t="s">
+        <v>548</v>
+      </c>
+    </row>
+    <row r="121" spans="1:2">
+      <c r="A121" t="s">
+        <v>2</v>
+      </c>
+      <c r="B121" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="122" spans="1:2">
+      <c r="A122" t="s">
+        <v>4</v>
+      </c>
+      <c r="B122" t="s">
+        <v>549</v>
+      </c>
+    </row>
+    <row r="123" spans="1:2">
+      <c r="A123" t="s">
+        <v>2</v>
+      </c>
+      <c r="B123" t="s">
+        <v>550</v>
+      </c>
+    </row>
+    <row r="124" spans="1:2">
+      <c r="A124" t="s">
+        <v>2</v>
+      </c>
+      <c r="B124" t="s">
+        <v>551</v>
+      </c>
+    </row>
+    <row r="125" spans="1:2">
+      <c r="A125" t="s">
+        <v>2</v>
+      </c>
+      <c r="B125" t="s">
+        <v>552</v>
+      </c>
+    </row>
+    <row r="126" spans="1:2">
+      <c r="A126" t="s">
+        <v>2</v>
+      </c>
+      <c r="B126" t="s">
+        <v>553</v>
+      </c>
+    </row>
+    <row r="127" spans="1:2">
+      <c r="A127" t="s">
+        <v>2</v>
+      </c>
+      <c r="B127" t="s">
+        <v>554</v>
+      </c>
+    </row>
+    <row r="128" spans="1:2">
+      <c r="A128" t="s">
+        <v>2</v>
+      </c>
+      <c r="B128" t="s">
+        <v>555</v>
+      </c>
+    </row>
+    <row r="129" spans="1:2">
+      <c r="A129" t="s">
+        <v>2</v>
+      </c>
+      <c r="B129" t="s">
+        <v>556</v>
+      </c>
+    </row>
+    <row r="130" spans="1:2" ht="180">
+      <c r="A130" t="s">
+        <v>2</v>
+      </c>
+      <c r="B130" s="2" t="s">
+        <v>475</v>
+      </c>
+    </row>
+    <row r="131" spans="1:2">
+      <c r="A131" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="132" spans="1:2">
+      <c r="A132" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="133" spans="1:2">
+      <c r="A133" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="134" spans="1:2">
+      <c r="A134" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="135" spans="1:2">
+      <c r="A135" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="136" spans="1:2">
+      <c r="A136" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="137" spans="1:2">
+      <c r="A137" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="138" spans="1:2">
+      <c r="A138" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="139" spans="1:2">
+      <c r="A139" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="140" spans="1:2">
+      <c r="A140" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="141" spans="1:2">
+      <c r="A141" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="142" spans="1:2">
+      <c r="A142" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="143" spans="1:2">
+      <c r="A143" t="s">
+        <v>2</v>
+      </c>
+      <c r="B143" t="s">
+        <v>557</v>
+      </c>
+    </row>
+    <row r="144" spans="1:2">
+      <c r="A144" t="s">
+        <v>2</v>
+      </c>
+      <c r="B144" t="s">
+        <v>558</v>
+      </c>
+    </row>
+    <row r="145" spans="1:2">
+      <c r="A145" t="s">
+        <v>2</v>
+      </c>
+      <c r="B145" t="s">
+        <v>484</v>
+      </c>
+    </row>
+    <row r="146" spans="1:2">
+      <c r="A146" t="s">
+        <v>13</v>
+      </c>
+      <c r="B146" s="3" t="s">
+        <v>559</v>
+      </c>
+    </row>
+    <row r="147" spans="1:2">
+      <c r="A147" t="s">
+        <v>4</v>
+      </c>
+      <c r="B147" s="7" t="s">
+        <v>560</v>
+      </c>
+    </row>
+    <row r="148" spans="1:2">
+      <c r="A148" t="s">
+        <v>4</v>
+      </c>
+      <c r="B148" t="s">
+        <v>561</v>
+      </c>
+    </row>
+    <row r="149" spans="1:2">
+      <c r="A149" t="s">
+        <v>2</v>
+      </c>
+      <c r="B149" t="s">
+        <v>562</v>
+      </c>
+    </row>
+    <row r="150" spans="1:2">
+      <c r="A150" t="s">
+        <v>2</v>
+      </c>
+      <c r="B150" t="s">
+        <v>563</v>
+      </c>
+    </row>
+    <row r="151" spans="1:2">
+      <c r="A151" t="s">
+        <v>4</v>
+      </c>
+      <c r="B151" t="s">
+        <v>564</v>
+      </c>
+    </row>
+    <row r="152" spans="1:2">
+      <c r="A152" t="s">
+        <v>2</v>
+      </c>
+      <c r="B152" t="s">
+        <v>565</v>
+      </c>
+    </row>
+    <row r="153" spans="1:2">
+      <c r="A153" t="s">
+        <v>2</v>
+      </c>
+      <c r="B153" t="s">
+        <v>566</v>
+      </c>
+    </row>
+    <row r="154" spans="1:2">
+      <c r="A154" t="s">
+        <v>2</v>
+      </c>
+      <c r="B154" t="s">
+        <v>567</v>
+      </c>
+    </row>
+    <row r="155" spans="1:2">
+      <c r="A155" t="s">
+        <v>4</v>
+      </c>
+      <c r="B155" t="s">
+        <v>569</v>
+      </c>
+    </row>
+    <row r="156" spans="1:2">
+      <c r="A156" t="s">
+        <v>2</v>
+      </c>
+      <c r="B156" t="s">
+        <v>568</v>
+      </c>
+    </row>
+    <row r="157" spans="1:2">
+      <c r="A157" t="s">
+        <v>2</v>
+      </c>
+      <c r="B157" t="s">
+        <v>484</v>
+      </c>
+    </row>
+    <row r="158" spans="1:2">
+      <c r="A158" t="s">
+        <v>13</v>
+      </c>
+      <c r="B158" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="159" spans="1:2">
+      <c r="A159" t="s">
+        <v>4</v>
+      </c>
+      <c r="B159" t="s">
+        <v>570</v>
+      </c>
+    </row>
+    <row r="160" spans="1:2">
+      <c r="A160" t="s">
+        <v>2</v>
+      </c>
+      <c r="B160" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="161" spans="1:2">
+      <c r="A161" t="s">
+        <v>2</v>
+      </c>
+      <c r="B161" t="s">
+        <v>484</v>
+      </c>
+    </row>
+    <row r="162" spans="1:2">
+      <c r="A162" t="s">
+        <v>13</v>
+      </c>
+      <c r="B162" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="163" spans="1:2">
+      <c r="A163" t="s">
+        <v>4</v>
+      </c>
+      <c r="B163" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="164" spans="1:2">
+      <c r="A164" t="s">
+        <v>2</v>
+      </c>
+      <c r="B164" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="165" spans="1:2">
+      <c r="A165" t="s">
+        <v>2</v>
+      </c>
+      <c r="B165" t="s">
+        <v>484</v>
+      </c>
+    </row>
+    <row r="166" spans="1:2">
+      <c r="A166" t="s">
+        <v>13</v>
+      </c>
+      <c r="B166" t="s">
+        <v>142</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="2" type="noConversion"/>
+  <hyperlinks>
+    <hyperlink ref="B13" r:id="rId1" xr:uid="{D9095DA6-4FB3-3E4D-BA09-A1CE936EDE60}"/>
+    <hyperlink ref="B16" r:id="rId2" xr:uid="{B2C1A08E-7E9F-3347-BE49-1EBFEC8203D6}"/>
+    <hyperlink ref="B19" r:id="rId3" xr:uid="{7B7094D5-904B-6243-AE18-639FCAF73573}"/>
+    <hyperlink ref="B22" r:id="rId4" xr:uid="{DC2F17C5-C168-7D4E-B3A3-D3184EE355A4}"/>
+    <hyperlink ref="B40" r:id="rId5" xr:uid="{0DBD1E02-D501-6F47-8235-B1EF430E6425}"/>
+    <hyperlink ref="B49" r:id="rId6" xr:uid="{65D86518-B361-C046-AA07-A7B023153E57}"/>
+    <hyperlink ref="B52" r:id="rId7" xr:uid="{C5836BD4-5EF4-F74A-8A97-5B8177650909}"/>
+    <hyperlink ref="B55" r:id="rId8" xr:uid="{83C99206-622F-3B48-89FA-CFD98D67A3D7}"/>
+    <hyperlink ref="B69" r:id="rId9" xr:uid="{D3DED111-D9FB-BB45-920B-0F4E6EB248F3}"/>
+    <hyperlink ref="B90" r:id="rId10" xr:uid="{239878BF-DFA5-DE4C-B568-A96D2227C65B}"/>
+    <hyperlink ref="B104" r:id="rId11" xr:uid="{9E2A6E74-DD39-4549-BDA8-74C7392F213C}"/>
+    <hyperlink ref="B119" r:id="rId12" xr:uid="{7858FB2A-1866-344E-8FCF-B7D4EC6E02B7}"/>
+    <hyperlink ref="B146" r:id="rId13" xr:uid="{47C04396-0651-ED4F-BB37-6687D5607853}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
📝 ADD : LG AI(BG)
</commit_message>
<xml_diff>
--- a/ai-gate/copy.xlsx
+++ b/ai-gate/copy.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="10727"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EC172FE6-AE50-E24D-AC0A-BDF6AD20994E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9DDA9A7C-59AD-454A-A2EA-25E8E93E9E7B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="34560" windowHeight="21580" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="34560" windowHeight="21580" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="sample" sheetId="1" r:id="rId1"/>
@@ -14,13 +14,14 @@
     <sheet name="BE_FR" sheetId="5" r:id="rId4"/>
     <sheet name="TN_FR" sheetId="6" r:id="rId5"/>
     <sheet name="SK" sheetId="8" r:id="rId6"/>
+    <sheet name="BG" sheetId="9" r:id="rId7"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1809" uniqueCount="575">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2105" uniqueCount="675">
   <si>
     <t>Type</t>
   </si>
@@ -27600,6 +27601,447 @@
       </rPr>
       <t>ou nasiakavosti.</t>
     </r>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Една жена преминава, когато светлината се включва автоматично. На екрана се появява надпис „Сензитивност“.
+Мъж и жена се прегръщат, когато се активира високоговорителят на XBOOM, придружен от думата  „Разбиране“.
+Мъж седи тъжно на шофьорската седалка. Появява се логото на LG AI с надпис "Грижа".
+По телевизията се излъчва футболен мач. LG AI реагира с гласово взаимодействие. Отдолу се показва фразата „За вашия възхитителен живот“.
+XBOOM, телевизорът и семейство, седнало на дивана с кучето си, се появяват в един кадър.
+Майка и син използват заедно пералната машина. Появява се фразата „За вашия безпроблемен живот“.
+Сцените на майката и сина, близък план на AI Wash и мъж, който използва лаптопа LG gram, се наслагват в един кадър, като се появява фразата „За безпроблемен живот“.
+Мъж и жена седят на предните седалки на автомобил. Логото на LG AI се появява между тях, заедно с фразата „За вашия живот с грижа“.
+Човек влиза в офис с кучето си. Пречиствателят на въздуха се включва.
+Финален кадър: бял фон с логото на LG AI и фразата „Интелегентност с грижа за ВАС“.</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>&lt;span class="gradient-text" data-tp="copy"&gt;Affectionate Intelligence&lt;/span&gt; за ВАС</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>В LG си задаваме въпроса: за какво трябва да съществува AI? &lt;br&gt;
+              След дълъг размисъл намерихме своя отговор. &lt;br&gt;&lt;br&gt;
+              За нас AI е нещо повече от изкуствен интелект - това е интелигентност с обич и грижа. &lt;br&gt;&lt;br&gt;
+              Тъй като AI става част от нашето ежедневие, &lt;br&gt;
+              той трябва да помогне за създаването на по-добър живот, който всички заслужаваме. &lt;br&gt;&lt;br&gt;
+              Ето защо AI на LG започва с обич към ВАС чрез &lt;br&gt;
+              сензитивност и разбиране, както и грижа за живота ви.
+              &lt;strong&gt;Открий как животът е хубав с  LG AI&lt;/strong&gt;</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Превъртете надолу иконата</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Прекрасен живот</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Безпроблемен живот</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Живот с грижа</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>LG AI разбира вашия живот и надгражда преживяванията, за да създаде  живот, изпълнен с прекрасни моменти.</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Мъж и жена седят на дивана и гледат футболно предаване на телевизор LG в хола. 
+Сцената се премества и мъжът и жената се прегръщат.
+Камерата се фокусира върху LG XBOOM до тях.</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>За вашия прекрасен живот</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>https://www.lg.com/bg/oled-evo</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>LG OLED evo AI продукти- фронтален изглед</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Научете повече</t>
+  </si>
+  <si>
+    <t>https://www.lg.com/bg/oled-tv</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>LG OLED AI продукти -фронтален изглед</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>https://www.lg.com/bg/qned-tv</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>LG QNED AI продукти- фронтален изглед</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>https://www.lg.com/bg/nanocell-tv</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>LG NanoCell AI продукти- фронтален изглед</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>LG AI усеща вашите нужди и представя решения, чрез които да направи живота ви безгрижен и според избрания ритъм.</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Майка и син използват заедно пералнята с LG AI, като завъртат копчето, за да активират функцията AI Wash. В същата сцена се появява мъж, който използва лаптоп LG gram.</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>За вашия  безпроблемен живот</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>https://www.lg.com/bg/lg-washtower</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>LG WashTower AI продукт- фронтален изглед</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>https://www.lg.com/bg/peralni-mashini/lg-f4wr513sbw</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>LG Washing Machine AI продукт- фронтален изглед</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>https://www.lg.com/bg/hladilnitzi/lg-gsgv81pyll</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>LG InstaView AI продукт- фронтален изглед</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>LG AI се грижи за вас, вашето пространство и за планетата, за да направи живота ви безгрижен.</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>В офиса влиза мъж с каишка за куче. Мъжът на шофьорската седалка изглежда тъжен, когато LG AI му показва семейна снимка. Дисплеят на автомобила е показан в близък план, докато LG AI изважда карта и се връща към спомен.</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>За вашия живот с грижа</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>https://www.lg.com/bg/klimatichna-tehnika/lg-p12snd</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>LG DUALCOOL AI продукт с фронтален изглед</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>ADAS vision система със страничен изглед</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Взаимодействие на потребителя със сензорен интерфейс, задвижван от мултимодално HMI решение с изкуствен интелект, избор на меню за кафе с подкана от асистент с изкуствен интелект.</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>ТВ</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Аудио</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Бяла техника</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Климатична техника</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>&lt;picture&gt;
+                        &lt;source srcset="./assets/image/ai-gate-image-product-category-tv-eyebrow-logo-desktop.svg" media="(min-width: 769px)"&gt;
+                        &lt;source srcset="./assets/image/ai-gate-image-product-category-tv-eyebrow-logo-mobile.svg" media="(max-width: 768px)"&gt;
+                        &lt;img src="./assets/image/ai-gate-image-product-category-tv-eyebrow-logo-mobile.svg" alt="ТВ" class="eyebrow-logo" loading="lazy"&gt;
+                      &lt;/picture&gt;
+                      Evolves to satisfy your every entertainment need</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Телевизорът с изкуствен интелект на LG научава предпочитанията ви за гледане и разбира начина ви на живот, за да оптимизира всеки аспект на телевизионното ви изживяване, създавайки идеално персонализирано забавление точно за вас.</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Над LG Magic Remote се показват функции като AI Chatbot, AI Picture Wizard и AI Sound Wizard.</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Запознайте се със следващо поколение &lt;br&gt;
+                          LG AI TV</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>https://www.lg.com/bg/televizori/ai-tv</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Научно-фантастично съдържание се възпроизвежда на екрана на OLED телевизор LG. В лявата част на екрана е разположен интерфейсът на AI Chatbot. Потребителят съобщава на чатбота, че екранът е твърде тъмен, и чатботът предлага решения на искането.</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Жена пее с микрофон със слушалки, с LG α11 AI Processor за подобряване на звука</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Две свързани сцени с LG AI Magic Remote пред телевизор - първата показва научнофантастична сцена, а втората - начален екран с персонализирано съдържание</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>*Функциите с изкуствен интелект на LG използват обучени алгоритми, базирани на дълбоко обучение, за увеличаване на мащаба на изображенията и смесване на звука в реално време.</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>**Всички телевизори LG webOS 24 разполагат с функция AI Customization, с изключение на тези без сензори за светлина.</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>&lt;picture&gt;
+                        &lt;source srcset="./assets/image/ai-gate-image-product-category-audio-eyebrow-logo-desktop.svg" media="(min-width: 769px)"&gt;
+                        &lt;source srcset="./assets/image/ai-gate-image-product-category-audio-eyebrow-logo-mobile.svg" media="(max-width: 768px)"&gt;
+                        &lt;img src="./assets/image/ai-gate-image-product-category-audio-eyebrow-logo-mobile.svg" alt="Аудио" class="eyebrow-logo" loading="lazy"&gt;
+                      &lt;/picture&gt;
+                      Звук, който звучи по най-правилния начин</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>LG xboom AI анализира и настройва звука, за да отговаря на жанра и пространството. Чрез AI осветлението, което подобрява обстановката и хармонизира с музиката, можете да се насладите на звук и атмосфера по уникален начин.</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Жена и мъж се прегръщат в хола, а до тях е включен високоговорителят на XBOOM.</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Наслаждавайте се на ново звуково преживяване с &lt;br&gt;
+                          LG xboom AI</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>LG XBOOM говорител с AI звукови режими включва Bass Boost, Voice Enhance и Standard.</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>AI Звук</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t xml:space="preserve">LG XBOOM говорител с AI осветелние, което се адаптира към глас, околна среда и парти режим. </t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>AI Осветление</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>AI Калибриране</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Високоговорител LG XBOOM, поставен на маса в стая в червени тонове, със стени с решетъчни шарки и модерни мебели.</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>*Този продукт все още не е наличен</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>&lt;picture&gt;
+                        &lt;source srcset="./assets/image/ai-gate-image-product-category-appliances-eyebrow-logo-desktop.svg" media="(min-width: 769px)"&gt;
+                        &lt;source srcset="./assets/image/ai-gate-image-product-category-appliances-eyebrow-logo-mobile.svg" media="(max-width: 768px)"&gt;
+                        &lt;img src="./assets/image/ai-gate-image-product-category-appliances-eyebrow-logo-mobile.svg" alt="Бяла техника" class="eyebrow-logo" loading="lazy"&gt;
+                      &lt;/picture&gt;
+                      Освобождаване от обемите пране</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>LG WashTower AI разпознава какво перете, за да осигури оптимизирано изпиране за чувствителни тъкани, като ви гарантира, че без усилие ще усъвършенствате всяко зареждане, всеки път.</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Вградени пералня и сушилня LG в модерно перално помещение с дървени шкафове и пейки за сядане.</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Открийте нов начин на живот с &lt;br&gt;
+                          LG AI Core Tech</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>https://www.lg.com/bg/peralni-mashini/lg-aidd</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Ръчно регулиране на цикъла на пране AI на пералната машина LG с помощта на интелигентен контролен диск</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>AI Пране</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Потребител, който избира AI Dry цикъл на сушилнята LG с помощта на цифровия контролен диск.</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>AI Сушене</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>*Този продукт ще бъде пуснат поетапно в избрани страни.</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>**Активира се сензорът за AI, когато товарът е под 6 kg.</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>***Измиването с AI трябва да се използва само с подобни видове тъкани [не всички тъкани се разпознават] и подходящ перилен препарат.</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>****AI Dry се предлага само за зареждания под 5 кг с тъкани със същите нива на абсорбция на влага.</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>&lt;picture&gt;
+                        &lt;source srcset="./assets/image/ai-gate-image-product-category-air-conditioning-eyebrow-logo-desktop.svg" media="(min-width: 769px)"&gt;
+                        &lt;source srcset="./assets/image/ai-gate-image-product-category-air-conditioning-eyebrow-logo-mobile.svg" media="(max-width: 768px)"&gt;
+                        &lt;img src="./assets/image/ai-gate-image-product-category-air-conditioning-eyebrow-logo-mobile.svg" alt="Климатична техника" class="eyebrow-logo" loading="lazy"&gt;
+                      &lt;/picture&gt;
+                      Комфорт с перфектно охлаждане</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>LG DUALCOOL AI се грижи за оптимален въздух, като ви осигурява комфорт и същевременно оптимизира енергийната ефективност, за да спести разходи. С LG AI Air се наслаждавайте на перфектно охлаждане за вашия комфорт.</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Инверторният климатик LG DUAL охлажда модерна всекидневна, в която жена е седнала на дивана, благодарение на технологията ThinQ AI.</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Оптимизиран комфорт с &lt;br&gt;
+                          LG AI Air</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Жена релаксира в смарт всекидневна, докато климатикът LG AI автоматично регулира температурата, въздушния поток и влажността.</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>AI Въздух</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Интерфейс на смартфон, показващ графика на потреблението на енергия пред климатик LG, с подчертан AI kW Manager за ефективен мониторинг на енергията.</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>*AI Air може да се управлява с дистанционно управление и ThinQ.</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>**AI Air се предлага в режими на охлаждане и отопление.</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>***По време на използване на AI Air обемът на въздуха и посоката на вятъра се регулират автоматично в зависимост от ситуацията, а AI Air се изключва при промяна на посоката на вятъра.</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>****Когато AI Air е активиран, радарният сензор открива местоположението на обекта и автоматично активира директния/непосредствения вятър.</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>*****Разстоянието на засичане на радарния сензор е до 5 м, като е възможно да има разлики в разстоянието на засичане в зависимост от средата на инсталиране и използване на продукта.</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>******Тази функция работи само с модели, които имат радарни сензори.</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>ThinQ® прави управлението да се случва лесно</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Приложение а за вашите интелигентни уреди и устройства, LG ThinQ предоставя контрол и удобство на ръка разстояние, за да ви помогне да опростите живота си и да се наслаждавате на домашния уют.</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>https://www.lg.com/bg/elektrodomakinski-uredi/thinq</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Човек държи смартфон, в който е отворено приложението LG ThinQ, и управлява  домашни устройства, докато пие кафе.</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Смартфонът показва приложението LG ThinQ за управление на фурната LG InstaView Slide-In Range, което позволява ефективна поддръжка на продукта в кухнята.</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Ефективна продуктова поддръжка</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Чрез приложението LG ThinQ проверявайте своя уред от LG, изтегляйте нови цикли, наблюдавайте използването  и много други.</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Повече за LG Affectionate Intelligence</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t xml:space="preserve">LG Electronics поддържа акредитация за киберсигурност с графика за цифрова сигурност. </t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>LG укрепва лидерството си в областта на киберсигурността с акредитацията на KOLAS за тестване на киберсигурността на IoT.</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Посетители разглеждат извития LED дисплей на LG, представящ слогана „Life's Good 24/7“ на технологично изложение.</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>LG представя на CES 2025 най-новите си иновации, задвижвани от „Аffectionate Intelligence“</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Говорител, който представя B2B решения с изкуствен интелект на сцената на събитие на LG.</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>LG представя един ден от живота с „Аffectionate Intelligence“ на световната премиера на LG</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
 </sst>
@@ -35620,4 +36062,1256 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A991E548-02F4-F043-A91A-3C844B35EB11}">
+  <dimension ref="A1:B166"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="17"/>
+  <cols>
+    <col min="1" max="1" width="15" customWidth="1"/>
+    <col min="2" max="2" width="120" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" s="1" customFormat="1">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" ht="234">
+      <c r="A2" t="s">
+        <v>2</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>575</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2">
+      <c r="A3" t="s">
+        <v>4</v>
+      </c>
+      <c r="B3" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2">
+      <c r="A4" t="s">
+        <v>313</v>
+      </c>
+      <c r="B4" t="s">
+        <v>576</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" ht="144">
+      <c r="A5" t="s">
+        <v>2</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>577</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2">
+      <c r="A6" t="s">
+        <v>4</v>
+      </c>
+      <c r="B6" t="s">
+        <v>578</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2">
+      <c r="A7" t="s">
+        <v>2</v>
+      </c>
+      <c r="B7" t="s">
+        <v>579</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2">
+      <c r="A8" t="s">
+        <v>2</v>
+      </c>
+      <c r="B8" t="s">
+        <v>580</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2">
+      <c r="A9" t="s">
+        <v>2</v>
+      </c>
+      <c r="B9" t="s">
+        <v>581</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2">
+      <c r="A10" t="s">
+        <v>2</v>
+      </c>
+      <c r="B10" t="s">
+        <v>582</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" ht="54">
+      <c r="A11" t="s">
+        <v>2</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>583</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2">
+      <c r="A12" t="s">
+        <v>2</v>
+      </c>
+      <c r="B12" t="s">
+        <v>584</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2">
+      <c r="A13" t="s">
+        <v>13</v>
+      </c>
+      <c r="B13" s="3" t="s">
+        <v>585</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2">
+      <c r="A14" t="s">
+        <v>4</v>
+      </c>
+      <c r="B14" t="s">
+        <v>586</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2">
+      <c r="A15" t="s">
+        <v>2</v>
+      </c>
+      <c r="B15" t="s">
+        <v>587</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2">
+      <c r="A16" t="s">
+        <v>13</v>
+      </c>
+      <c r="B16" s="3" t="s">
+        <v>588</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2">
+      <c r="A17" t="s">
+        <v>4</v>
+      </c>
+      <c r="B17" t="s">
+        <v>589</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2">
+      <c r="A18" t="s">
+        <v>2</v>
+      </c>
+      <c r="B18" t="s">
+        <v>587</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2">
+      <c r="A19" t="s">
+        <v>13</v>
+      </c>
+      <c r="B19" s="3" t="s">
+        <v>590</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2">
+      <c r="A20" t="s">
+        <v>4</v>
+      </c>
+      <c r="B20" t="s">
+        <v>591</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2">
+      <c r="A21" t="s">
+        <v>2</v>
+      </c>
+      <c r="B21" t="s">
+        <v>587</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2">
+      <c r="A22" t="s">
+        <v>13</v>
+      </c>
+      <c r="B22" s="3" t="s">
+        <v>592</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2">
+      <c r="A23" t="s">
+        <v>4</v>
+      </c>
+      <c r="B23" t="s">
+        <v>593</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2">
+      <c r="A24" t="s">
+        <v>2</v>
+      </c>
+      <c r="B24" t="s">
+        <v>587</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2">
+      <c r="A25" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="26" spans="1:2">
+      <c r="A26" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="27" spans="1:2">
+      <c r="A27" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="28" spans="1:2">
+      <c r="A28" t="s">
+        <v>2</v>
+      </c>
+      <c r="B28" t="s">
+        <v>594</v>
+      </c>
+    </row>
+    <row r="29" spans="1:2">
+      <c r="A29" t="s">
+        <v>2</v>
+      </c>
+      <c r="B29" t="s">
+        <v>595</v>
+      </c>
+    </row>
+    <row r="30" spans="1:2">
+      <c r="A30" t="s">
+        <v>2</v>
+      </c>
+      <c r="B30" t="s">
+        <v>596</v>
+      </c>
+    </row>
+    <row r="31" spans="1:2">
+      <c r="A31" t="s">
+        <v>13</v>
+      </c>
+      <c r="B31" s="3" t="s">
+        <v>597</v>
+      </c>
+    </row>
+    <row r="32" spans="1:2">
+      <c r="A32" t="s">
+        <v>4</v>
+      </c>
+      <c r="B32" t="s">
+        <v>598</v>
+      </c>
+    </row>
+    <row r="33" spans="1:2">
+      <c r="A33" t="s">
+        <v>2</v>
+      </c>
+      <c r="B33" t="s">
+        <v>587</v>
+      </c>
+    </row>
+    <row r="34" spans="1:2">
+      <c r="A34" t="s">
+        <v>13</v>
+      </c>
+      <c r="B34" s="3" t="s">
+        <v>599</v>
+      </c>
+    </row>
+    <row r="35" spans="1:2">
+      <c r="A35" t="s">
+        <v>4</v>
+      </c>
+      <c r="B35" t="s">
+        <v>600</v>
+      </c>
+    </row>
+    <row r="36" spans="1:2">
+      <c r="A36" t="s">
+        <v>2</v>
+      </c>
+      <c r="B36" t="s">
+        <v>587</v>
+      </c>
+    </row>
+    <row r="37" spans="1:2">
+      <c r="A37" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="38" spans="1:2">
+      <c r="A38" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="39" spans="1:2">
+      <c r="A39" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="40" spans="1:2">
+      <c r="A40" t="s">
+        <v>13</v>
+      </c>
+      <c r="B40" s="3" t="s">
+        <v>601</v>
+      </c>
+    </row>
+    <row r="41" spans="1:2">
+      <c r="A41" t="s">
+        <v>4</v>
+      </c>
+      <c r="B41" t="s">
+        <v>602</v>
+      </c>
+    </row>
+    <row r="42" spans="1:2">
+      <c r="A42" t="s">
+        <v>2</v>
+      </c>
+      <c r="B42" t="s">
+        <v>587</v>
+      </c>
+    </row>
+    <row r="43" spans="1:2">
+      <c r="A43" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="44" spans="1:2">
+      <c r="A44" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="45" spans="1:2">
+      <c r="A45" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="46" spans="1:2">
+      <c r="A46" t="s">
+        <v>2</v>
+      </c>
+      <c r="B46" t="s">
+        <v>603</v>
+      </c>
+    </row>
+    <row r="47" spans="1:2">
+      <c r="A47" t="s">
+        <v>2</v>
+      </c>
+      <c r="B47" t="s">
+        <v>604</v>
+      </c>
+    </row>
+    <row r="48" spans="1:2">
+      <c r="A48" t="s">
+        <v>2</v>
+      </c>
+      <c r="B48" t="s">
+        <v>605</v>
+      </c>
+    </row>
+    <row r="49" spans="1:2">
+      <c r="A49" t="s">
+        <v>13</v>
+      </c>
+      <c r="B49" s="3" t="s">
+        <v>606</v>
+      </c>
+    </row>
+    <row r="50" spans="1:2">
+      <c r="A50" t="s">
+        <v>4</v>
+      </c>
+      <c r="B50" t="s">
+        <v>607</v>
+      </c>
+    </row>
+    <row r="51" spans="1:2">
+      <c r="A51" t="s">
+        <v>2</v>
+      </c>
+      <c r="B51" t="s">
+        <v>587</v>
+      </c>
+    </row>
+    <row r="52" spans="1:2">
+      <c r="A52" t="s">
+        <v>13</v>
+      </c>
+      <c r="B52" s="3" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="53" spans="1:2">
+      <c r="A53" t="s">
+        <v>4</v>
+      </c>
+      <c r="B53" t="s">
+        <v>608</v>
+      </c>
+    </row>
+    <row r="54" spans="1:2">
+      <c r="A54" t="s">
+        <v>2</v>
+      </c>
+      <c r="B54" t="s">
+        <v>587</v>
+      </c>
+    </row>
+    <row r="55" spans="1:2">
+      <c r="A55" t="s">
+        <v>13</v>
+      </c>
+      <c r="B55" s="3" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="56" spans="1:2">
+      <c r="A56" t="s">
+        <v>4</v>
+      </c>
+      <c r="B56" t="s">
+        <v>609</v>
+      </c>
+    </row>
+    <row r="57" spans="1:2">
+      <c r="A57" t="s">
+        <v>2</v>
+      </c>
+      <c r="B57" t="s">
+        <v>587</v>
+      </c>
+    </row>
+    <row r="58" spans="1:2">
+      <c r="A58" t="s">
+        <v>2</v>
+      </c>
+      <c r="B58" t="s">
+        <v>610</v>
+      </c>
+    </row>
+    <row r="59" spans="1:2">
+      <c r="A59" t="s">
+        <v>2</v>
+      </c>
+      <c r="B59" t="s">
+        <v>611</v>
+      </c>
+    </row>
+    <row r="60" spans="1:2">
+      <c r="A60" t="s">
+        <v>2</v>
+      </c>
+      <c r="B60" t="s">
+        <v>612</v>
+      </c>
+    </row>
+    <row r="61" spans="1:2">
+      <c r="A61" t="s">
+        <v>2</v>
+      </c>
+      <c r="B61" t="s">
+        <v>613</v>
+      </c>
+    </row>
+    <row r="62" spans="1:2">
+      <c r="A62" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="63" spans="1:2" ht="162">
+      <c r="A63" t="s">
+        <v>2</v>
+      </c>
+      <c r="B63" s="2" t="s">
+        <v>614</v>
+      </c>
+    </row>
+    <row r="64" spans="1:2">
+      <c r="A64" t="s">
+        <v>4</v>
+      </c>
+      <c r="B64" t="s">
+        <v>610</v>
+      </c>
+    </row>
+    <row r="65" spans="1:2">
+      <c r="A65" t="s">
+        <v>2</v>
+      </c>
+      <c r="B65" t="s">
+        <v>615</v>
+      </c>
+    </row>
+    <row r="66" spans="1:2">
+      <c r="A66" t="s">
+        <v>4</v>
+      </c>
+      <c r="B66" t="s">
+        <v>616</v>
+      </c>
+    </row>
+    <row r="67" spans="1:2" ht="36">
+      <c r="A67" t="s">
+        <v>2</v>
+      </c>
+      <c r="B67" s="2" t="s">
+        <v>617</v>
+      </c>
+    </row>
+    <row r="68" spans="1:2">
+      <c r="A68" t="s">
+        <v>2</v>
+      </c>
+      <c r="B68" t="s">
+        <v>587</v>
+      </c>
+    </row>
+    <row r="69" spans="1:2">
+      <c r="A69" t="s">
+        <v>13</v>
+      </c>
+      <c r="B69" s="3" t="s">
+        <v>618</v>
+      </c>
+    </row>
+    <row r="70" spans="1:2">
+      <c r="A70" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="71" spans="1:2">
+      <c r="A71" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="72" spans="1:2">
+      <c r="A72" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="73" spans="1:2">
+      <c r="A73" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="74" spans="1:2">
+      <c r="A74" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="75" spans="1:2">
+      <c r="A75" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="76" spans="1:2">
+      <c r="A76" t="s">
+        <v>4</v>
+      </c>
+      <c r="B76" t="s">
+        <v>619</v>
+      </c>
+    </row>
+    <row r="77" spans="1:2">
+      <c r="A77" t="s">
+        <v>2</v>
+      </c>
+      <c r="B77" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="78" spans="1:2">
+      <c r="A78" t="s">
+        <v>4</v>
+      </c>
+      <c r="B78" t="s">
+        <v>620</v>
+      </c>
+    </row>
+    <row r="79" spans="1:2">
+      <c r="A79" t="s">
+        <v>2</v>
+      </c>
+      <c r="B79" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="80" spans="1:2">
+      <c r="A80" t="s">
+        <v>4</v>
+      </c>
+      <c r="B80" t="s">
+        <v>621</v>
+      </c>
+    </row>
+    <row r="81" spans="1:2">
+      <c r="A81" t="s">
+        <v>2</v>
+      </c>
+      <c r="B81" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="82" spans="1:2">
+      <c r="A82" t="s">
+        <v>2</v>
+      </c>
+      <c r="B82" t="s">
+        <v>622</v>
+      </c>
+    </row>
+    <row r="83" spans="1:2">
+      <c r="A83" t="s">
+        <v>2</v>
+      </c>
+      <c r="B83" t="s">
+        <v>623</v>
+      </c>
+    </row>
+    <row r="84" spans="1:2" ht="162">
+      <c r="A84" t="s">
+        <v>2</v>
+      </c>
+      <c r="B84" s="2" t="s">
+        <v>624</v>
+      </c>
+    </row>
+    <row r="85" spans="1:2">
+      <c r="A85" t="s">
+        <v>4</v>
+      </c>
+      <c r="B85" t="s">
+        <v>611</v>
+      </c>
+    </row>
+    <row r="86" spans="1:2">
+      <c r="A86" t="s">
+        <v>2</v>
+      </c>
+      <c r="B86" t="s">
+        <v>625</v>
+      </c>
+    </row>
+    <row r="87" spans="1:2">
+      <c r="A87" t="s">
+        <v>4</v>
+      </c>
+      <c r="B87" t="s">
+        <v>626</v>
+      </c>
+    </row>
+    <row r="88" spans="1:2" ht="36">
+      <c r="A88" t="s">
+        <v>2</v>
+      </c>
+      <c r="B88" s="2" t="s">
+        <v>627</v>
+      </c>
+    </row>
+    <row r="89" spans="1:2">
+      <c r="A89" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="90" spans="1:2">
+      <c r="A90" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="91" spans="1:2">
+      <c r="A91" t="s">
+        <v>4</v>
+      </c>
+      <c r="B91" t="s">
+        <v>628</v>
+      </c>
+    </row>
+    <row r="92" spans="1:2">
+      <c r="A92" t="s">
+        <v>2</v>
+      </c>
+      <c r="B92" t="s">
+        <v>629</v>
+      </c>
+    </row>
+    <row r="93" spans="1:2">
+      <c r="A93" t="s">
+        <v>4</v>
+      </c>
+      <c r="B93" t="s">
+        <v>630</v>
+      </c>
+    </row>
+    <row r="94" spans="1:2">
+      <c r="A94" t="s">
+        <v>2</v>
+      </c>
+      <c r="B94" t="s">
+        <v>631</v>
+      </c>
+    </row>
+    <row r="95" spans="1:2">
+      <c r="A95" t="s">
+        <v>4</v>
+      </c>
+      <c r="B95" t="s">
+        <v>633</v>
+      </c>
+    </row>
+    <row r="96" spans="1:2">
+      <c r="A96" t="s">
+        <v>2</v>
+      </c>
+      <c r="B96" t="s">
+        <v>632</v>
+      </c>
+    </row>
+    <row r="97" spans="1:2">
+      <c r="A97" t="s">
+        <v>2</v>
+      </c>
+      <c r="B97" t="s">
+        <v>634</v>
+      </c>
+    </row>
+    <row r="98" spans="1:2" ht="162">
+      <c r="A98" t="s">
+        <v>2</v>
+      </c>
+      <c r="B98" s="2" t="s">
+        <v>635</v>
+      </c>
+    </row>
+    <row r="99" spans="1:2">
+      <c r="A99" t="s">
+        <v>4</v>
+      </c>
+      <c r="B99" t="s">
+        <v>612</v>
+      </c>
+    </row>
+    <row r="100" spans="1:2">
+      <c r="A100" t="s">
+        <v>2</v>
+      </c>
+      <c r="B100" t="s">
+        <v>636</v>
+      </c>
+    </row>
+    <row r="101" spans="1:2">
+      <c r="A101" t="s">
+        <v>4</v>
+      </c>
+      <c r="B101" t="s">
+        <v>637</v>
+      </c>
+    </row>
+    <row r="102" spans="1:2" ht="36">
+      <c r="A102" t="s">
+        <v>2</v>
+      </c>
+      <c r="B102" s="2" t="s">
+        <v>638</v>
+      </c>
+    </row>
+    <row r="103" spans="1:2">
+      <c r="A103" t="s">
+        <v>2</v>
+      </c>
+      <c r="B103" t="s">
+        <v>587</v>
+      </c>
+    </row>
+    <row r="104" spans="1:2">
+      <c r="A104" t="s">
+        <v>13</v>
+      </c>
+      <c r="B104" s="3" t="s">
+        <v>639</v>
+      </c>
+    </row>
+    <row r="105" spans="1:2">
+      <c r="A105" t="s">
+        <v>4</v>
+      </c>
+      <c r="B105" t="s">
+        <v>640</v>
+      </c>
+    </row>
+    <row r="106" spans="1:2">
+      <c r="A106" t="s">
+        <v>2</v>
+      </c>
+      <c r="B106" t="s">
+        <v>641</v>
+      </c>
+    </row>
+    <row r="107" spans="1:2">
+      <c r="A107" t="s">
+        <v>4</v>
+      </c>
+      <c r="B107" t="s">
+        <v>642</v>
+      </c>
+    </row>
+    <row r="108" spans="1:2">
+      <c r="A108" t="s">
+        <v>2</v>
+      </c>
+      <c r="B108" t="s">
+        <v>643</v>
+      </c>
+    </row>
+    <row r="109" spans="1:2">
+      <c r="A109" t="s">
+        <v>2</v>
+      </c>
+      <c r="B109" t="s">
+        <v>644</v>
+      </c>
+    </row>
+    <row r="110" spans="1:2">
+      <c r="A110" t="s">
+        <v>2</v>
+      </c>
+      <c r="B110" t="s">
+        <v>645</v>
+      </c>
+    </row>
+    <row r="111" spans="1:2">
+      <c r="A111" t="s">
+        <v>2</v>
+      </c>
+      <c r="B111" t="s">
+        <v>646</v>
+      </c>
+    </row>
+    <row r="112" spans="1:2">
+      <c r="A112" t="s">
+        <v>2</v>
+      </c>
+      <c r="B112" t="s">
+        <v>647</v>
+      </c>
+    </row>
+    <row r="113" spans="1:2" ht="162">
+      <c r="A113" t="s">
+        <v>2</v>
+      </c>
+      <c r="B113" s="2" t="s">
+        <v>648</v>
+      </c>
+    </row>
+    <row r="114" spans="1:2">
+      <c r="A114" t="s">
+        <v>4</v>
+      </c>
+      <c r="B114" t="s">
+        <v>613</v>
+      </c>
+    </row>
+    <row r="115" spans="1:2">
+      <c r="A115" t="s">
+        <v>2</v>
+      </c>
+      <c r="B115" t="s">
+        <v>649</v>
+      </c>
+    </row>
+    <row r="116" spans="1:2">
+      <c r="A116" t="s">
+        <v>4</v>
+      </c>
+      <c r="B116" t="s">
+        <v>650</v>
+      </c>
+    </row>
+    <row r="117" spans="1:2" ht="36">
+      <c r="A117" t="s">
+        <v>2</v>
+      </c>
+      <c r="B117" s="2" t="s">
+        <v>651</v>
+      </c>
+    </row>
+    <row r="118" spans="1:2">
+      <c r="A118" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="119" spans="1:2">
+      <c r="A119" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="120" spans="1:2">
+      <c r="A120" t="s">
+        <v>4</v>
+      </c>
+      <c r="B120" t="s">
+        <v>652</v>
+      </c>
+    </row>
+    <row r="121" spans="1:2">
+      <c r="A121" t="s">
+        <v>2</v>
+      </c>
+      <c r="B121" t="s">
+        <v>653</v>
+      </c>
+    </row>
+    <row r="122" spans="1:2">
+      <c r="A122" t="s">
+        <v>4</v>
+      </c>
+      <c r="B122" t="s">
+        <v>654</v>
+      </c>
+    </row>
+    <row r="123" spans="1:2">
+      <c r="A123" t="s">
+        <v>2</v>
+      </c>
+      <c r="B123" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="124" spans="1:2">
+      <c r="A124" t="s">
+        <v>2</v>
+      </c>
+      <c r="B124" t="s">
+        <v>655</v>
+      </c>
+    </row>
+    <row r="125" spans="1:2">
+      <c r="A125" t="s">
+        <v>2</v>
+      </c>
+      <c r="B125" t="s">
+        <v>656</v>
+      </c>
+    </row>
+    <row r="126" spans="1:2">
+      <c r="A126" t="s">
+        <v>2</v>
+      </c>
+      <c r="B126" t="s">
+        <v>657</v>
+      </c>
+    </row>
+    <row r="127" spans="1:2">
+      <c r="A127" t="s">
+        <v>2</v>
+      </c>
+      <c r="B127" t="s">
+        <v>658</v>
+      </c>
+    </row>
+    <row r="128" spans="1:2">
+      <c r="A128" t="s">
+        <v>2</v>
+      </c>
+      <c r="B128" t="s">
+        <v>659</v>
+      </c>
+    </row>
+    <row r="129" spans="1:2">
+      <c r="A129" t="s">
+        <v>2</v>
+      </c>
+      <c r="B129" t="s">
+        <v>660</v>
+      </c>
+    </row>
+    <row r="130" spans="1:2">
+      <c r="A130" t="s">
+        <v>2</v>
+      </c>
+      <c r="B130" s="2"/>
+    </row>
+    <row r="131" spans="1:2">
+      <c r="A131" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="132" spans="1:2">
+      <c r="A132" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="133" spans="1:2">
+      <c r="A133" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="134" spans="1:2">
+      <c r="A134" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="135" spans="1:2">
+      <c r="A135" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="136" spans="1:2">
+      <c r="A136" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="137" spans="1:2">
+      <c r="A137" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="138" spans="1:2">
+      <c r="A138" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="139" spans="1:2">
+      <c r="A139" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="140" spans="1:2">
+      <c r="A140" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="141" spans="1:2">
+      <c r="A141" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="142" spans="1:2">
+      <c r="A142" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="143" spans="1:2">
+      <c r="A143" t="s">
+        <v>2</v>
+      </c>
+      <c r="B143" t="s">
+        <v>661</v>
+      </c>
+    </row>
+    <row r="144" spans="1:2">
+      <c r="A144" t="s">
+        <v>2</v>
+      </c>
+      <c r="B144" t="s">
+        <v>662</v>
+      </c>
+    </row>
+    <row r="145" spans="1:2">
+      <c r="A145" t="s">
+        <v>2</v>
+      </c>
+      <c r="B145" t="s">
+        <v>587</v>
+      </c>
+    </row>
+    <row r="146" spans="1:2">
+      <c r="A146" t="s">
+        <v>13</v>
+      </c>
+      <c r="B146" s="3" t="s">
+        <v>663</v>
+      </c>
+    </row>
+    <row r="147" spans="1:2">
+      <c r="A147" t="s">
+        <v>4</v>
+      </c>
+      <c r="B147" t="s">
+        <v>664</v>
+      </c>
+    </row>
+    <row r="148" spans="1:2">
+      <c r="A148" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="149" spans="1:2">
+      <c r="A149" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="150" spans="1:2">
+      <c r="A150" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="151" spans="1:2">
+      <c r="A151" t="s">
+        <v>4</v>
+      </c>
+      <c r="B151" t="s">
+        <v>665</v>
+      </c>
+    </row>
+    <row r="152" spans="1:2">
+      <c r="A152" t="s">
+        <v>2</v>
+      </c>
+      <c r="B152" t="s">
+        <v>666</v>
+      </c>
+    </row>
+    <row r="153" spans="1:2">
+      <c r="A153" t="s">
+        <v>2</v>
+      </c>
+      <c r="B153" t="s">
+        <v>667</v>
+      </c>
+    </row>
+    <row r="154" spans="1:2">
+      <c r="A154" t="s">
+        <v>2</v>
+      </c>
+      <c r="B154" t="s">
+        <v>668</v>
+      </c>
+    </row>
+    <row r="155" spans="1:2">
+      <c r="A155" t="s">
+        <v>4</v>
+      </c>
+      <c r="B155" t="s">
+        <v>669</v>
+      </c>
+    </row>
+    <row r="156" spans="1:2">
+      <c r="A156" t="s">
+        <v>2</v>
+      </c>
+      <c r="B156" t="s">
+        <v>670</v>
+      </c>
+    </row>
+    <row r="157" spans="1:2">
+      <c r="A157" t="s">
+        <v>2</v>
+      </c>
+      <c r="B157" t="s">
+        <v>587</v>
+      </c>
+    </row>
+    <row r="158" spans="1:2">
+      <c r="A158" t="s">
+        <v>13</v>
+      </c>
+      <c r="B158" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="159" spans="1:2">
+      <c r="A159" t="s">
+        <v>4</v>
+      </c>
+      <c r="B159" t="s">
+        <v>671</v>
+      </c>
+    </row>
+    <row r="160" spans="1:2">
+      <c r="A160" t="s">
+        <v>2</v>
+      </c>
+      <c r="B160" t="s">
+        <v>672</v>
+      </c>
+    </row>
+    <row r="161" spans="1:2">
+      <c r="A161" t="s">
+        <v>2</v>
+      </c>
+      <c r="B161" t="s">
+        <v>587</v>
+      </c>
+    </row>
+    <row r="162" spans="1:2">
+      <c r="A162" t="s">
+        <v>13</v>
+      </c>
+      <c r="B162" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="163" spans="1:2">
+      <c r="A163" t="s">
+        <v>4</v>
+      </c>
+      <c r="B163" t="s">
+        <v>673</v>
+      </c>
+    </row>
+    <row r="164" spans="1:2">
+      <c r="A164" t="s">
+        <v>2</v>
+      </c>
+      <c r="B164" t="s">
+        <v>674</v>
+      </c>
+    </row>
+    <row r="165" spans="1:2">
+      <c r="A165" t="s">
+        <v>2</v>
+      </c>
+      <c r="B165" t="s">
+        <v>587</v>
+      </c>
+    </row>
+    <row r="166" spans="1:2">
+      <c r="A166" t="s">
+        <v>13</v>
+      </c>
+      <c r="B166" t="s">
+        <v>142</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="2" type="noConversion"/>
+  <hyperlinks>
+    <hyperlink ref="B13" r:id="rId1" xr:uid="{5B01F28E-0A55-594E-94C5-5C81AD1C43E6}"/>
+    <hyperlink ref="B16" r:id="rId2" xr:uid="{90B219FD-0D2E-2842-968D-050A0B1ADBF7}"/>
+    <hyperlink ref="B19" r:id="rId3" xr:uid="{BF54A870-5159-E24D-B344-D68CA27194B8}"/>
+    <hyperlink ref="B22" r:id="rId4" xr:uid="{564D10A8-DC3F-864E-A663-D03439698A51}"/>
+    <hyperlink ref="B31" r:id="rId5" xr:uid="{223BE860-1155-E84A-891B-13209FBD68C1}"/>
+    <hyperlink ref="B34" r:id="rId6" xr:uid="{3834B966-88C5-9745-A351-A06179BF7FE8}"/>
+    <hyperlink ref="B40" r:id="rId7" xr:uid="{F7ED3F57-484D-F84B-8703-1361220D4B64}"/>
+    <hyperlink ref="B49" r:id="rId8" xr:uid="{15330C5B-D989-F644-8B84-17C618A55C7B}"/>
+    <hyperlink ref="B52" r:id="rId9" xr:uid="{816926B0-D7D3-D74C-9E67-9C54B16996B4}"/>
+    <hyperlink ref="B55" r:id="rId10" xr:uid="{0F8E9FD9-FB4D-9C4C-8299-391F5D7AFC1B}"/>
+    <hyperlink ref="B69" r:id="rId11" xr:uid="{E11A81D7-8798-7047-88B8-445D374A06D3}"/>
+    <hyperlink ref="B104" r:id="rId12" xr:uid="{04E234A5-B841-1F4E-93C7-4353D245DCDE}"/>
+    <hyperlink ref="B146" r:id="rId13" xr:uid="{D24EA7E2-E0A9-0341-AE3E-E3CBCD1FC65E}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>
+</worksheet>
 </file>
</xml_diff>